<commit_message>
added abs for PMC
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="449" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{744367AC-89EA-47A7-80A8-7356E30D38F8}"/>
+  <xr:revisionPtr revIDLastSave="450" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5543BEAD-19CA-4177-AFE6-173518DC31BD}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AY2023-2024 Sem 2" sheetId="3" state="hidden" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="445">
   <si>
     <t>Fill in as much of the green boxes as possible. Ideally, this would be before you have finished your visitors travel dates (just to avoid double booking).</t>
   </si>
@@ -1442,6 +1442,9 @@
   </si>
   <si>
     <t>Leornard Henckel</t>
+  </si>
+  <si>
+    <t>In today's complex, increasingly interconnected world, old paradigms for supporting decision making under uncertainty are falling short of the needs of decision-makers.  Typically, a wide range of factors are at play, each overseen by specialists who rely on large, complex models to oversee and make forecasts for their particular part of the system.  A single overarching model for the whole system is infeasible and rapidly becomes outdated as matters evolve.  The Integrating Decision Support System was developed to provide a robust statistical underpinning for decision support systems in such circumstances. The IDSS is a transparent and principled method for drawing together evidence from multiple expert domains, including the relevant uncertainties, and turning these into usable insights that can support decision centres in evaluating and comparing the range of policy options at their disposal.</t>
   </si>
 </sst>
 </file>
@@ -7175,7 +7178,7 @@
       <c r="X14" s="15"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26">
         <v>46155</v>
       </c>
@@ -7238,7 +7241,7 @@
         <v>394</v>
       </c>
       <c r="J16" t="s">
-        <v>395</v>
+        <v>444</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -7277,6 +7280,7 @@
     <hyperlink ref="K14" r:id="rId14" xr:uid="{F5CA8E46-DA4D-40A2-B71F-BC8C3D5249DB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
updated PMC speakers time
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="450" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5543BEAD-19CA-4177-AFE6-173518DC31BD}"/>
+  <xr:revisionPtr revIDLastSave="458" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B4BB872-9EFA-4F7A-A37A-1B4A774269D3}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AY2023-2024 Sem 2" sheetId="3" state="hidden" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="448">
   <si>
     <t>Fill in as much of the green boxes as possible. Ideally, this would be before you have finished your visitors travel dates (just to avoid double booking).</t>
   </si>
@@ -1445,6 +1445,15 @@
   </si>
   <si>
     <t>In today's complex, increasingly interconnected world, old paradigms for supporting decision making under uncertainty are falling short of the needs of decision-makers.  Typically, a wide range of factors are at play, each overseen by specialists who rely on large, complex models to oversee and make forecasts for their particular part of the system.  A single overarching model for the whole system is infeasible and rapidly becomes outdated as matters evolve.  The Integrating Decision Support System was developed to provide a robust statistical underpinning for decision support systems in such circumstances. The IDSS is a transparent and principled method for drawing together evidence from multiple expert domains, including the relevant uncertainties, and turning these into usable insights that can support decision centres in evaluating and comparing the range of policy options at their disposal.</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/citations?hl=en&amp;user=z9-sxWMAAAAJ&amp;view_op=list_works&amp;sortby=pubdate</t>
+  </si>
+  <si>
+    <t>https://warwick.ac.uk/fac/sci/statistics/staff/academic-research/barons/</t>
+  </si>
+  <si>
+    <t>10am</t>
   </si>
 </sst>
 </file>
@@ -1985,7 +1994,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="172">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -2272,6 +2281,7 @@
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -7209,6 +7219,12 @@
       <c r="J15" s="129" t="s">
         <v>390</v>
       </c>
+      <c r="K15" s="172" t="s">
+        <v>445</v>
+      </c>
+      <c r="M15" t="s">
+        <v>446</v>
+      </c>
       <c r="X15" s="20"/>
       <c r="Y15" s="18"/>
     </row>
@@ -7217,7 +7233,7 @@
         <v>46176</v>
       </c>
       <c r="B16" t="s">
-        <v>190</v>
+        <v>447</v>
       </c>
       <c r="C16" s="26" t="s">
         <v>391</v>
@@ -7278,9 +7294,10 @@
     <hyperlink ref="K11" r:id="rId12" xr:uid="{460148DF-9775-4F8A-91F3-89030F1FC4E8}"/>
     <hyperlink ref="M14" r:id="rId13" xr:uid="{8D133BC0-60B4-4F75-84B7-5C8F4452AAD4}"/>
     <hyperlink ref="K14" r:id="rId14" xr:uid="{F5CA8E46-DA4D-40A2-B71F-BC8C3D5249DB}"/>
+    <hyperlink ref="K15" r:id="rId15" xr:uid="{E8AE30CF-C39D-45BD-88FA-74BD7A1EDBAB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="0" orientation="portrait" r:id="rId15"/>
+  <pageSetup paperSize="0" orientation="portrait" r:id="rId16"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
updated for new sem
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="458" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B4BB872-9EFA-4F7A-A37A-1B4A774269D3}"/>
+  <xr:revisionPtr revIDLastSave="477" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6266729F-4B00-43CE-BFB7-427447B7C737}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AY2023-2024 Sem 2" sheetId="3" state="hidden" r:id="rId1"/>
     <sheet name="AY2024-2025 Sem 1" sheetId="1" state="hidden" r:id="rId2"/>
     <sheet name="AY2024-2025 Sem 2" sheetId="6" state="hidden" r:id="rId3"/>
     <sheet name="AY2025-2026 Sem 1" sheetId="7" state="hidden" r:id="rId4"/>
-    <sheet name="AY2025-2026 Sem 2" sheetId="9" r:id="rId5"/>
-    <sheet name="AY2026-2027 Sem 1" sheetId="10" r:id="rId6"/>
-    <sheet name="Possbile speaker (reserve list)" sheetId="4" r:id="rId7"/>
-    <sheet name="Open dates" sheetId="8" r:id="rId8"/>
-    <sheet name="Printed A2002" sheetId="5" state="hidden" r:id="rId9"/>
+    <sheet name="AY2026-2027 Sem 1" sheetId="10" r:id="rId5"/>
+    <sheet name="AY2026-2027 Sem 2" sheetId="12" r:id="rId6"/>
+    <sheet name="AY2025-2026 Sem 2" sheetId="9" r:id="rId7"/>
+    <sheet name="Possbile speaker (reserve list)" sheetId="4" r:id="rId8"/>
+    <sheet name="Open dates" sheetId="8" r:id="rId9"/>
+    <sheet name="Printed A2002" sheetId="5" state="hidden" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="448">
   <si>
     <t>Fill in as much of the green boxes as possible. Ideally, this would be before you have finished your visitors travel dates (just to avoid double booking).</t>
   </si>
@@ -1090,6 +1091,15 @@
     <t>https://www.tcd.ie/scss/people/academic-staff/dangelos/ ; https://sites.google.com/view/silviadangelo/home</t>
   </si>
   <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>TBC</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
     <t>Eoin O’Brien</t>
   </si>
   <si>
@@ -1244,9 +1254,6 @@
     <t>The tipping of the Atlantic Meridional Overturning Circulation (AMOC) to a ‘shutdown’ state due to changes in the freshwater forcing of the ocean is of particular interest and concern due to its widespread ramifications, including a dramatic climatic shift for much of Europe. A clear understanding of how such a shutdown would unfold requires analyses of models from across the complexity spectrum. For example, detailed simulations of sophisticated Earth System Models have identified scenarios of ‘fragmented’ tipping towards a complete shutdown of AMOC, in which deep-water formation first ceases in the Labrador Sea before ceasing in the Nordic Seas. Here, we study a simple ocean box model with two polar boxes designed to represent deep-water formation at these two distinct sites. A bifurcation analysis reveals how, depending on the differences of freshwater and thermal forcing between the two polar boxes, transitions to ‘partial shutdown’ states are possible. Our results shed light on the nature of the tipping of AMOC and clarify dynamical features observed in more sophisticated models.</t>
   </si>
   <si>
-    <t>May</t>
-  </si>
-  <si>
     <t>Florian Faucher</t>
   </si>
   <si>
@@ -1284,6 +1291,15 @@
 </t>
   </si>
   <si>
+    <t>https://scholar.google.com/citations?hl=en&amp;user=z9-sxWMAAAAJ&amp;view_op=list_works&amp;sortby=pubdate</t>
+  </si>
+  <si>
+    <t>https://warwick.ac.uk/fac/sci/statistics/staff/academic-research/barons/</t>
+  </si>
+  <si>
+    <t>10am</t>
+  </si>
+  <si>
     <t>June</t>
   </si>
   <si>
@@ -1297,10 +1313,7 @@
 </t>
   </si>
   <si>
-    <t>TBC</t>
-  </si>
-  <si>
-    <t>Open</t>
+    <t>In today's complex, increasingly interconnected world, old paradigms for supporting decision making under uncertainty are falling short of the needs of decision-makers.  Typically, a wide range of factors are at play, each overseen by specialists who rely on large, complex models to oversee and make forecasts for their particular part of the system.  A single overarching model for the whole system is infeasible and rapidly becomes outdated as matters evolve.  The Integrating Decision Support System was developed to provide a robust statistical underpinning for decision support systems in such circumstances. The IDSS is a transparent and principled method for drawing together evidence from multiple expert domains, including the relevant uncertainties, and turning these into usable insights that can support decision centres in evaluating and comparing the range of policy options at their disposal.</t>
   </si>
   <si>
     <t>This is a just a place for those who are interested but that dont have a specific date in mind. (Ideally, a couple of these are people that we could invite with relatively short notice to fill missing slots.)</t>
@@ -1442,18 +1455,6 @@
   </si>
   <si>
     <t>Leornard Henckel</t>
-  </si>
-  <si>
-    <t>In today's complex, increasingly interconnected world, old paradigms for supporting decision making under uncertainty are falling short of the needs of decision-makers.  Typically, a wide range of factors are at play, each overseen by specialists who rely on large, complex models to oversee and make forecasts for their particular part of the system.  A single overarching model for the whole system is infeasible and rapidly becomes outdated as matters evolve.  The Integrating Decision Support System was developed to provide a robust statistical underpinning for decision support systems in such circumstances. The IDSS is a transparent and principled method for drawing together evidence from multiple expert domains, including the relevant uncertainties, and turning these into usable insights that can support decision centres in evaluating and comparing the range of policy options at their disposal.</t>
-  </si>
-  <si>
-    <t>https://scholar.google.com/citations?hl=en&amp;user=z9-sxWMAAAAJ&amp;view_op=list_works&amp;sortby=pubdate</t>
-  </si>
-  <si>
-    <t>https://warwick.ac.uk/fac/sci/statistics/staff/academic-research/barons/</t>
-  </si>
-  <si>
-    <t>10am</t>
   </si>
 </sst>
 </file>
@@ -1463,7 +1464,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2322,9 +2323,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2362,7 +2363,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2468,7 +2469,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2610,7 +2611,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2619,7 +2620,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7958562-D4BB-4776-9668-682A6F2E2AD0}">
   <dimension ref="A1:Y20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="11.140625" customWidth="1"/>
@@ -2644,7 +2645,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2655,7 +2656,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="30">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2732,7 +2733,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="13.5" customHeight="1">
       <c r="A3" s="2">
         <v>45317</v>
       </c>
@@ -2799,7 +2800,7 @@
       <c r="X3" s="13"/>
       <c r="Y3" s="13"/>
     </row>
-    <row r="4" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="13.5" customHeight="1">
       <c r="A4" s="2">
         <v>45323</v>
       </c>
@@ -2862,7 +2863,7 @@
       <c r="X4" s="13"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25">
       <c r="A5" s="2">
         <v>45324</v>
       </c>
@@ -2923,7 +2924,7 @@
       <c r="X5" s="13"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="12.75" customHeight="1">
       <c r="A6" s="2">
         <v>45331</v>
       </c>
@@ -2990,7 +2991,7 @@
       <c r="X6" s="13"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25">
       <c r="A7" s="2">
         <v>45338</v>
       </c>
@@ -3059,7 +3060,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="15" customHeight="1">
       <c r="A8" s="2">
         <v>45345</v>
       </c>
@@ -3126,7 +3127,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="16.5" customHeight="1">
       <c r="A9" s="2">
         <v>45359</v>
       </c>
@@ -3179,7 +3180,7 @@
       <c r="X9" s="13"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25">
       <c r="A10" s="2">
         <v>45366</v>
       </c>
@@ -3248,7 +3249,7 @@
       <c r="X10" s="13"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15" customHeight="1">
       <c r="A11" s="2">
         <v>45379</v>
       </c>
@@ -3309,7 +3310,7 @@
       <c r="X11" s="13"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="13.5" customHeight="1">
       <c r="A12" s="2">
         <v>45386</v>
       </c>
@@ -3372,7 +3373,7 @@
       <c r="X12" s="13"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="16.5" customHeight="1">
       <c r="A13" s="2">
         <v>45387</v>
       </c>
@@ -3441,7 +3442,7 @@
       <c r="X13" s="13"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1">
       <c r="A14" s="2">
         <v>45394</v>
       </c>
@@ -3502,7 +3503,7 @@
       <c r="X14" s="13"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="17.25" customHeight="1">
       <c r="A15" s="2">
         <v>45398</v>
       </c>
@@ -3571,7 +3572,7 @@
       <c r="X15" s="13"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25">
       <c r="A16" s="2">
         <v>45401</v>
       </c>
@@ -3634,7 +3635,7 @@
       <c r="X16" s="18"/>
       <c r="Y16" s="18"/>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25">
       <c r="A17" s="4">
         <v>45421</v>
       </c>
@@ -3705,7 +3706,7 @@
       <c r="X17" s="18"/>
       <c r="Y17" s="18"/>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25">
       <c r="A18" s="26">
         <v>45474</v>
       </c>
@@ -3756,7 +3757,7 @@
       <c r="X18" s="18"/>
       <c r="Y18" s="18"/>
     </row>
-    <row r="19" spans="1:25" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:25" ht="17.25" customHeight="1" thickBot="1">
       <c r="A19" s="26">
         <v>45505</v>
       </c>
@@ -3807,7 +3808,7 @@
       <c r="X19" s="18"/>
       <c r="Y19" s="18"/>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25">
       <c r="A20" s="26"/>
       <c r="B20" s="26"/>
       <c r="C20" s="26"/>
@@ -3846,10 +3847,325 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2BB5C5F-5790-4A91-A6E8-8841719DA1FC}">
+  <dimension ref="A2:I20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" customWidth="1"/>
+    <col min="7" max="7" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.42578125" customWidth="1"/>
+    <col min="9" max="9" width="64.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:9" ht="23.25">
+      <c r="A2" s="91" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="18.75">
+      <c r="A3" s="79" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="37.5">
+      <c r="A5" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="80" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="80" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="80" t="s">
+        <v>137</v>
+      </c>
+      <c r="E5" s="80" t="s">
+        <v>189</v>
+      </c>
+      <c r="F5" s="80" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="80" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="82" t="s">
+        <v>444</v>
+      </c>
+      <c r="I5" s="81" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="18.75">
+      <c r="A6" s="92">
+        <v>45694</v>
+      </c>
+      <c r="B6" s="92" t="s">
+        <v>190</v>
+      </c>
+      <c r="C6" s="92" t="s">
+        <v>191</v>
+      </c>
+      <c r="D6" s="93" t="s">
+        <v>278</v>
+      </c>
+      <c r="E6" s="93">
+        <v>2</v>
+      </c>
+      <c r="F6" s="85" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="85" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" s="85"/>
+      <c r="I6" s="84" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="18.75">
+      <c r="A7" s="83">
+        <v>45708</v>
+      </c>
+      <c r="B7" s="83" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7" s="83" t="s">
+        <v>191</v>
+      </c>
+      <c r="D7" s="94" t="s">
+        <v>278</v>
+      </c>
+      <c r="E7" s="94">
+        <v>4</v>
+      </c>
+      <c r="F7" s="87" t="s">
+        <v>194</v>
+      </c>
+      <c r="G7" s="87" t="s">
+        <v>195</v>
+      </c>
+      <c r="H7" s="87" t="s">
+        <v>78</v>
+      </c>
+      <c r="I7" s="86" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="18.75">
+      <c r="A8" s="83">
+        <v>45722</v>
+      </c>
+      <c r="B8" s="83" t="s">
+        <v>190</v>
+      </c>
+      <c r="C8" s="83" t="s">
+        <v>198</v>
+      </c>
+      <c r="D8" s="94" t="s">
+        <v>278</v>
+      </c>
+      <c r="E8" s="94">
+        <v>6</v>
+      </c>
+      <c r="F8" s="87" t="s">
+        <v>199</v>
+      </c>
+      <c r="G8" s="87" t="s">
+        <v>68</v>
+      </c>
+      <c r="H8" s="87" t="s">
+        <v>200</v>
+      </c>
+      <c r="I8" s="86"/>
+    </row>
+    <row r="9" spans="1:9" ht="18.75">
+      <c r="A9" s="83">
+        <v>45735</v>
+      </c>
+      <c r="B9" s="83" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="83" t="s">
+        <v>198</v>
+      </c>
+      <c r="D9" s="94" t="s">
+        <v>388</v>
+      </c>
+      <c r="E9" s="94">
+        <v>8</v>
+      </c>
+      <c r="F9" s="87" t="s">
+        <v>204</v>
+      </c>
+      <c r="G9" s="87" t="s">
+        <v>205</v>
+      </c>
+      <c r="H9" s="87" t="s">
+        <v>206</v>
+      </c>
+      <c r="I9" s="86" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="18.75">
+      <c r="A10" s="83">
+        <v>45744</v>
+      </c>
+      <c r="B10" s="83" t="s">
+        <v>190</v>
+      </c>
+      <c r="C10" s="83" t="s">
+        <v>198</v>
+      </c>
+      <c r="D10" s="94" t="s">
+        <v>214</v>
+      </c>
+      <c r="E10" s="94">
+        <v>9</v>
+      </c>
+      <c r="F10" s="87" t="s">
+        <v>222</v>
+      </c>
+      <c r="G10" s="87" t="s">
+        <v>223</v>
+      </c>
+      <c r="H10" s="87" t="s">
+        <v>224</v>
+      </c>
+      <c r="I10" s="86"/>
+    </row>
+    <row r="11" spans="1:9" ht="18.75">
+      <c r="A11" s="83">
+        <v>45750</v>
+      </c>
+      <c r="B11" s="83" t="s">
+        <v>190</v>
+      </c>
+      <c r="C11" s="83" t="s">
+        <v>209</v>
+      </c>
+      <c r="D11" s="94" t="s">
+        <v>278</v>
+      </c>
+      <c r="E11" s="94">
+        <v>10</v>
+      </c>
+      <c r="F11" s="87" t="s">
+        <v>445</v>
+      </c>
+      <c r="G11" s="87" t="s">
+        <v>68</v>
+      </c>
+      <c r="H11" s="87"/>
+      <c r="I11" s="86" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="18.75">
+      <c r="A12" s="83">
+        <v>45758</v>
+      </c>
+      <c r="B12" s="83" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="83" t="s">
+        <v>209</v>
+      </c>
+      <c r="D12" s="94" t="s">
+        <v>214</v>
+      </c>
+      <c r="E12" s="94">
+        <v>11</v>
+      </c>
+      <c r="F12" s="87" t="s">
+        <v>229</v>
+      </c>
+      <c r="G12" s="87" t="s">
+        <v>172</v>
+      </c>
+      <c r="H12" s="87" t="s">
+        <v>31</v>
+      </c>
+      <c r="I12" s="86" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="18.75">
+      <c r="A13" s="83">
+        <v>45764</v>
+      </c>
+      <c r="B13" s="83" t="s">
+        <v>190</v>
+      </c>
+      <c r="C13" s="83" t="s">
+        <v>209</v>
+      </c>
+      <c r="D13" s="94" t="s">
+        <v>278</v>
+      </c>
+      <c r="E13" s="94">
+        <v>12</v>
+      </c>
+      <c r="F13" s="87" t="s">
+        <v>446</v>
+      </c>
+      <c r="G13" s="87"/>
+      <c r="H13" s="87"/>
+      <c r="I13" s="86"/>
+    </row>
+    <row r="14" spans="1:9" ht="18.75">
+      <c r="A14" s="88">
+        <v>45771</v>
+      </c>
+      <c r="B14" s="88" t="s">
+        <v>190</v>
+      </c>
+      <c r="C14" s="88" t="s">
+        <v>209</v>
+      </c>
+      <c r="D14" s="95" t="s">
+        <v>278</v>
+      </c>
+      <c r="E14" s="95">
+        <v>13</v>
+      </c>
+      <c r="F14" s="90" t="s">
+        <v>447</v>
+      </c>
+      <c r="G14" s="90" t="s">
+        <v>77</v>
+      </c>
+      <c r="H14" s="90" t="s">
+        <v>124</v>
+      </c>
+      <c r="I14" s="89" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="20" spans="8:8" ht="18.75">
+      <c r="H20" s="79"/>
+    </row>
+  </sheetData>
+  <protectedRanges>
+    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A6:E13" name="Range3_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="A5:I5" name="Range4_1"/>
+    <protectedRange sqref="F6:I13" name="Range8_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A14" name="Range3_3"/>
+  </protectedRanges>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="11.140625" customWidth="1"/>
@@ -3874,7 +4190,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3885,7 +4201,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" ht="30.75" thickBot="1">
       <c r="A2" s="145" t="s">
         <v>3</v>
       </c>
@@ -3962,7 +4278,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15" customHeight="1">
       <c r="A3" s="2">
         <v>45548</v>
       </c>
@@ -4027,7 +4343,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15" customHeight="1">
       <c r="A4" s="2">
         <v>45555</v>
       </c>
@@ -4076,7 +4392,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="15" customHeight="1">
       <c r="A5" s="2">
         <v>45562</v>
       </c>
@@ -4125,7 +4441,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15" customHeight="1">
       <c r="A6" s="2">
         <v>45576</v>
       </c>
@@ -4174,7 +4490,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="15" customHeight="1">
       <c r="A7" s="2">
         <v>45583</v>
       </c>
@@ -4223,7 +4539,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="15" customHeight="1">
       <c r="A8" s="2">
         <v>45596</v>
       </c>
@@ -4272,7 +4588,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="15" customHeight="1">
       <c r="A9" s="2">
         <v>45604</v>
       </c>
@@ -4321,7 +4637,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15" customHeight="1">
       <c r="A10" s="2">
         <v>45611</v>
       </c>
@@ -4370,7 +4686,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15" customHeight="1">
       <c r="A11" s="2">
         <v>45625</v>
       </c>
@@ -4419,7 +4735,7 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25" ht="15" customHeight="1" thickBot="1">
       <c r="A12" s="4">
         <v>45632</v>
       </c>
@@ -4476,20 +4792,20 @@
       <c r="X12" s="20"/>
       <c r="Y12" s="18"/>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25">
       <c r="A13" s="26"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
       <c r="D13" s="26"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25">
       <c r="A14" s="26"/>
       <c r="B14" s="26"/>
       <c r="C14" s="26"/>
       <c r="D14" s="26"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -4501,59 +4817,59 @@
       <c r="I29" s="61"/>
       <c r="J29" s="61"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10">
       <c r="A31" s="60"/>
       <c r="B31" s="60"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10">
       <c r="A32" s="60"/>
       <c r="B32" s="60"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2">
       <c r="A33" s="60"/>
       <c r="B33" s="60"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2">
       <c r="A34" s="60"/>
       <c r="B34" s="60"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2">
       <c r="A35" s="60"/>
       <c r="B35" s="60"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2">
       <c r="A36" s="60"/>
       <c r="B36" s="60"/>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2">
       <c r="A37" s="60"/>
       <c r="B37" s="60"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2">
       <c r="A38" s="60"/>
       <c r="B38" s="60"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2">
       <c r="A39" s="60"/>
       <c r="B39" s="60"/>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2">
       <c r="A40" s="60"/>
       <c r="B40" s="60"/>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2">
       <c r="A41" s="60"/>
       <c r="B41" s="60"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2">
       <c r="A42" s="60"/>
       <c r="B42" s="60"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2">
       <c r="A43" s="60"/>
       <c r="B43" s="60"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2">
       <c r="A44" s="60"/>
       <c r="B44" s="60"/>
     </row>
@@ -4582,7 +4898,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12299A9A-6C0C-4F92-957E-FBFCB6211744}">
   <dimension ref="A1:Y45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="5.85546875" bestFit="1" customWidth="1"/>
@@ -4610,7 +4926,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4621,7 +4937,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" ht="27.75" customHeight="1" thickBot="1">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -4698,7 +5014,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15" customHeight="1">
       <c r="A3" s="2">
         <v>45694</v>
       </c>
@@ -4750,7 +5066,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="14.25" customHeight="1">
       <c r="A4" s="2">
         <v>45708</v>
       </c>
@@ -4808,7 +5124,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="14.25" customHeight="1">
       <c r="A5" s="2">
         <v>45722</v>
       </c>
@@ -4864,7 +5180,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="16.5" customHeight="1">
       <c r="A6" s="2">
         <v>45735</v>
       </c>
@@ -4920,7 +5236,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="18" customHeight="1">
       <c r="A7" s="2">
         <v>45750</v>
       </c>
@@ -4974,7 +5290,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="16.5" customHeight="1">
       <c r="A8" s="2">
         <v>45751</v>
       </c>
@@ -5033,7 +5349,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1">
       <c r="A9" s="2">
         <v>45757</v>
       </c>
@@ -5095,7 +5411,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1">
       <c r="A10" s="2">
         <v>45758</v>
       </c>
@@ -5149,7 +5465,7 @@
       <c r="X10" s="20"/>
       <c r="Y10" s="18"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1">
       <c r="A11" s="4">
         <v>45764</v>
       </c>
@@ -5209,7 +5525,7 @@
       <c r="X11" s="35"/>
       <c r="Y11" s="35"/>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1">
       <c r="A12" s="4">
         <v>45771</v>
       </c>
@@ -5270,7 +5586,7 @@
       <c r="X12" s="35"/>
       <c r="Y12" s="35"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1">
       <c r="A13" s="2">
         <v>45785</v>
       </c>
@@ -5323,7 +5639,7 @@
       <c r="X13" s="35"/>
       <c r="Y13" s="35"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1">
       <c r="A14" s="4">
         <v>45799</v>
       </c>
@@ -5369,7 +5685,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1">
       <c r="A15" s="4">
         <v>45805</v>
       </c>
@@ -5403,101 +5719,101 @@
         <v>250</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1">
       <c r="A16" s="75"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2">
       <c r="A17" s="26"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2">
       <c r="A18" s="26"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2">
       <c r="A19" s="26"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2">
       <c r="A20" s="75"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2">
       <c r="A21" s="26"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2">
       <c r="A22" s="75"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2">
       <c r="A23" s="26"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2">
       <c r="A24" s="26"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2">
       <c r="A25" s="26"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2">
       <c r="A26" s="26"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2">
       <c r="A27" s="26"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2">
       <c r="A28" s="26"/>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2">
       <c r="B31" s="60"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2">
       <c r="A32" s="60"/>
       <c r="B32" s="60"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2">
       <c r="A33" s="60"/>
       <c r="B33" s="60"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2">
       <c r="A34" s="60"/>
       <c r="B34" s="60"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2">
       <c r="A35" s="60"/>
       <c r="B35" s="60"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2">
       <c r="A36" s="60"/>
       <c r="B36" s="60"/>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2">
       <c r="A37" s="60"/>
       <c r="B37" s="60"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2">
       <c r="A38" s="60"/>
       <c r="B38" s="60"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2">
       <c r="A39" s="60"/>
       <c r="B39" s="60"/>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2">
       <c r="A40" s="60"/>
       <c r="B40" s="60"/>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2">
       <c r="A41" s="60"/>
       <c r="B41" s="60"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2">
       <c r="A42" s="60"/>
       <c r="B42" s="60"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2">
       <c r="A43" s="60"/>
       <c r="B43" s="60"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2">
       <c r="A44" s="60"/>
       <c r="B44" s="60"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2">
       <c r="A45" s="60"/>
     </row>
   </sheetData>
@@ -5522,7 +5838,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{243C2AD8-98F5-4435-96A3-1C2CAB922825}">
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
@@ -5549,7 +5865,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5560,7 +5876,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="30">
       <c r="A2" s="78" t="s">
         <v>3</v>
       </c>
@@ -5637,7 +5953,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" ht="15" customHeight="1" thickBot="1">
       <c r="A3" s="159">
         <v>45911</v>
       </c>
@@ -5700,7 +6016,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15" customHeight="1">
       <c r="A4" s="160">
         <v>45917</v>
       </c>
@@ -5769,7 +6085,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="15" customHeight="1">
       <c r="A5" s="160">
         <v>45926</v>
       </c>
@@ -5827,7 +6143,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15" customHeight="1">
       <c r="A6" s="160">
         <v>45939</v>
       </c>
@@ -5891,7 +6207,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="15" customHeight="1">
       <c r="A7" s="160">
         <v>45946</v>
       </c>
@@ -5948,7 +6264,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="15" customHeight="1">
       <c r="A8" s="160">
         <v>45953</v>
       </c>
@@ -6006,7 +6322,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="15" customHeight="1">
       <c r="A9" s="160">
         <v>45967</v>
       </c>
@@ -6068,7 +6384,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15" customHeight="1">
       <c r="A10" s="160">
         <v>45974</v>
       </c>
@@ -6131,7 +6447,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15" customHeight="1">
       <c r="A11" s="160">
         <v>45980</v>
       </c>
@@ -6182,7 +6498,7 @@
       <c r="X11" s="35"/>
       <c r="Y11" s="35"/>
     </row>
-    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1">
       <c r="A12" s="160">
         <f>A10+7</f>
         <v>45981</v>
@@ -6235,7 +6551,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25">
       <c r="A13" s="160">
         <v>45986</v>
       </c>
@@ -6271,7 +6587,7 @@
       <c r="M13" s="158"/>
       <c r="N13" s="158"/>
     </row>
-    <row r="14" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15" customHeight="1">
       <c r="A14" s="160">
         <v>45988</v>
       </c>
@@ -6326,7 +6642,7 @@
       <c r="X14" s="15"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25" ht="15" customHeight="1" thickBot="1">
       <c r="A15" s="161">
         <v>45995</v>
       </c>
@@ -6389,35 +6705,35 @@
       <c r="X15" s="15"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:25" ht="15" customHeight="1" thickBot="1">
       <c r="A16" s="26"/>
       <c r="B16" s="26"/>
       <c r="C16" s="26"/>
       <c r="X16" s="20"/>
       <c r="Y16" s="18"/>
     </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="15" customHeight="1">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
     </row>
-    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="15" customHeight="1">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
     </row>
-    <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="15" customHeight="1">
       <c r="A19" s="26"/>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
     </row>
-    <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:3" ht="15" customHeight="1"/>
+    <row r="21" spans="1:3" ht="15" customHeight="1"/>
+    <row r="22" spans="1:3" ht="15" customHeight="1"/>
+    <row r="23" spans="1:3" ht="15" customHeight="1"/>
+    <row r="24" spans="1:3" ht="15" customHeight="1"/>
+    <row r="25" spans="1:3" ht="15" customHeight="1"/>
+    <row r="26" spans="1:3" ht="15" customHeight="1"/>
   </sheetData>
   <protectedRanges>
     <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A3:E19" name="Range3_1"/>
@@ -6446,12 +6762,518 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F62D4156-0A06-4DBF-B1E7-3E12580121CB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A33E49C-EC2E-42B7-80E4-DD607C0B7A89}">
   <sheetPr>
-    <tabColor theme="9"/>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
+  <dimension ref="A1:Y13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="6" max="6" width="33.42578125" customWidth="1"/>
+    <col min="7" max="7" width="30.85546875" customWidth="1"/>
+    <col min="8" max="8" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.85546875" customWidth="1"/>
+    <col min="11" max="11" width="20.42578125" customWidth="1"/>
+    <col min="12" max="13" width="12.5703125" customWidth="1"/>
+    <col min="14" max="14" width="43.140625" customWidth="1"/>
+    <col min="15" max="15" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="36.5703125" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="39" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25" ht="15.75" thickBot="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="P1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="30.75" thickBot="1">
+      <c r="A2" s="64" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="76" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="63" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="78" t="s">
+        <v>137</v>
+      </c>
+      <c r="E2" s="64" t="s">
+        <v>189</v>
+      </c>
+      <c r="F2" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="141" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="142" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="143" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="140" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" s="144" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" s="66" t="s">
+        <v>14</v>
+      </c>
+      <c r="M2" s="66" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" s="67" t="s">
+        <v>16</v>
+      </c>
+      <c r="O2" s="68" t="s">
+        <v>17</v>
+      </c>
+      <c r="P2" s="66" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q2" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="R2" s="66" t="s">
+        <v>20</v>
+      </c>
+      <c r="S2" s="67" t="s">
+        <v>21</v>
+      </c>
+      <c r="T2" s="69" t="s">
+        <v>22</v>
+      </c>
+      <c r="U2" s="67" t="s">
+        <v>23</v>
+      </c>
+      <c r="V2" s="65" t="s">
+        <v>24</v>
+      </c>
+      <c r="W2" s="66" t="s">
+        <v>138</v>
+      </c>
+      <c r="X2" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y2" s="70" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" ht="15" customHeight="1">
+      <c r="A3" s="75">
+        <v>46275</v>
+      </c>
+      <c r="B3" s="77" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="29" t="str">
+        <f>TEXT(A3, "mmm")</f>
+        <v>Sep</v>
+      </c>
+      <c r="D3" s="55" t="str">
+        <f>TEXT(A3, "dddd")</f>
+        <v>Thursday</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="I3" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="J3" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="K3" s="73"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="35"/>
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="40"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="35"/>
+      <c r="U3" s="40"/>
+      <c r="V3" s="40"/>
+      <c r="W3" s="40"/>
+      <c r="X3" s="46"/>
+      <c r="Y3" s="44"/>
+    </row>
+    <row r="4" spans="1:25" ht="15.75" customHeight="1">
+      <c r="A4" s="75">
+        <f>A3+14</f>
+        <v>46289</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C4" s="26" t="str">
+        <f t="shared" ref="C4:C7" si="0">TEXT(A4, "mmm")</f>
+        <v>Sep</v>
+      </c>
+      <c r="D4" s="27" t="str">
+        <f t="shared" ref="D4:D8" si="1">TEXT(A4, "dddd")</f>
+        <v>Thursday</v>
+      </c>
+      <c r="E4">
+        <f>E3+2</f>
+        <v>3</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="I4" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="J4" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="K4" s="102"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="16"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="5"/>
+      <c r="W4" s="5"/>
+      <c r="X4" s="15"/>
+      <c r="Y4" s="13"/>
+    </row>
+    <row r="5" spans="1:25">
+      <c r="A5" s="75">
+        <f t="shared" ref="A5" si="2">A4+14</f>
+        <v>46303</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C5" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v>Oct</v>
+      </c>
+      <c r="D5" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>Thursday</v>
+      </c>
+      <c r="E5">
+        <f t="shared" ref="E5:E6" si="3">E4+2</f>
+        <v>5</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="I5" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="J5" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="K5" s="102"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="35"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="5"/>
+      <c r="S5" s="16"/>
+      <c r="T5" s="35"/>
+      <c r="U5" s="5"/>
+      <c r="V5" s="5"/>
+      <c r="W5" s="5"/>
+      <c r="X5" s="15"/>
+      <c r="Y5" s="13"/>
+    </row>
+    <row r="6" spans="1:25" ht="15.75" customHeight="1">
+      <c r="A6" s="75">
+        <f>A5+14</f>
+        <v>46317</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C6" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v>Oct</v>
+      </c>
+      <c r="D6" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>Thursday</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="I6" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="J6" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="K6" s="102"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="35"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="16"/>
+      <c r="T6" s="35"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="5"/>
+      <c r="X6" s="15"/>
+      <c r="Y6" s="13"/>
+    </row>
+    <row r="7" spans="1:25">
+      <c r="A7" s="75">
+        <f>A6+14</f>
+        <v>46331</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v>Nov</v>
+      </c>
+      <c r="D7" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>Thursday</v>
+      </c>
+      <c r="E7">
+        <f>E6+2</f>
+        <v>9</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="I7" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="J7" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="K7" s="102"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="35"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="16"/>
+      <c r="T7" s="35"/>
+      <c r="U7" s="5"/>
+      <c r="V7" s="5"/>
+      <c r="W7" s="5"/>
+      <c r="X7" s="15"/>
+      <c r="Y7" s="13"/>
+    </row>
+    <row r="8" spans="1:25">
+      <c r="A8" s="75">
+        <f>A7+14</f>
+        <v>46345</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>209</v>
+      </c>
+      <c r="D8" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>Thursday</v>
+      </c>
+      <c r="E8">
+        <v>11</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="I8" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="J8" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="K8" s="102"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="35"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="16"/>
+      <c r="T8" s="35"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="5"/>
+      <c r="W8" s="5"/>
+      <c r="X8" s="15"/>
+      <c r="Y8" s="13"/>
+    </row>
+    <row r="9" spans="1:25" ht="18.75" customHeight="1">
+      <c r="A9" s="75">
+        <v>46121</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>329</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="E9">
+        <v>13</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="I9" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="J9" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="K9" s="102"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="35"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="16"/>
+      <c r="T9" s="35"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+      <c r="X9" s="15"/>
+      <c r="Y9" s="13"/>
+    </row>
+    <row r="10" spans="1:25" ht="15.75" thickBot="1">
+      <c r="A10" s="26"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="X10" s="20"/>
+      <c r="Y10" s="18"/>
+    </row>
+    <row r="11" spans="1:25" ht="12.75" customHeight="1">
+      <c r="A11" s="26"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+    </row>
+    <row r="12" spans="1:25">
+      <c r="A12" s="26"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+    </row>
+    <row r="13" spans="1:25">
+      <c r="A13" s="26"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+    </row>
+  </sheetData>
+  <protectedRanges>
+    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A3:E13" name="Range3_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="A2:L2 N2:Y2" name="Range4_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="B/N8xqtMc7pXr3rfrr4k91A6IFAPX6lxEHUr9qsJ3yHA+MBnFuw+x27DjsTYKp86iL5C7QQh1TPFTQHueWpZbw==" saltValue="c0IR/echnZmip5yS1t29Rw==" spinCount="100000" sqref="T3:T9" name="Range6_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="BKDH3ki5lE3XQdc5qZnIH6o8wW8E0PkHgMZFCkv/XYDEa+b/qenui0oReDIqPDXHceUVJ+rEgU3I9CDBHraDYg==" saltValue="ruXqG4NOhhm7cSLor8wHfw==" spinCount="100000" sqref="O2:O9" name="Range7_1"/>
+    <protectedRange sqref="X10:Y10 F3:Y9" name="Range8_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="M2" name="Range4_1_1"/>
+  </protectedRanges>
+  <phoneticPr fontId="10" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5DF1960-42A2-4A6F-A85A-E44221287C02}">
+  <sheetPr>
+    <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:Y18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -6478,7 +7300,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6489,7 +7311,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="30.75">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -6566,9 +7388,9 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15" customHeight="1">
       <c r="A3" s="75">
-        <v>46051</v>
+        <v>46415</v>
       </c>
       <c r="B3" s="77" t="s">
         <v>190</v>
@@ -6590,14 +7412,14 @@
       <c r="G3" s="14" t="s">
         <v>328</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>200</v>
+      <c r="H3" s="14" t="s">
+        <v>328</v>
       </c>
       <c r="I3" s="98" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J3" s="98" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="K3" s="73"/>
       <c r="L3" s="40"/>
@@ -6615,40 +7437,40 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1">
       <c r="A4" s="75">
-        <f>A3+12</f>
-        <v>46063</v>
+        <f>A3+14</f>
+        <v>46429</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>331</v>
+        <v>190</v>
       </c>
       <c r="C4" s="26" t="str">
-        <f t="shared" ref="C4:C10" si="0">TEXT(A4, "mmm")</f>
+        <f t="shared" ref="C4:C7" si="0">TEXT(A4, "mmm")</f>
         <v>Feb</v>
       </c>
       <c r="D4" s="27" t="str">
-        <f t="shared" ref="D4:D10" si="1">TEXT(A4, "dddd")</f>
-        <v>Tuesday</v>
+        <f t="shared" ref="D4:D8" si="1">TEXT(A4, "dddd")</f>
+        <v>Thursday</v>
       </c>
       <c r="E4">
         <f>E3+2</f>
         <v>3</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>332</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>269</v>
+        <v>327</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>328</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>87</v>
+        <v>328</v>
       </c>
       <c r="I4" s="98" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J4" s="98" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="K4" s="102"/>
       <c r="L4" s="5"/>
@@ -6666,10 +7488,10 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="18.75" customHeight="1">
       <c r="A5" s="75">
-        <f>A4+16</f>
-        <v>46079</v>
+        <f t="shared" ref="A5" si="2">A4+14</f>
+        <v>46443</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>190</v>
@@ -6683,34 +7505,30 @@
         <v>Thursday</v>
       </c>
       <c r="E5">
-        <f t="shared" ref="E5:E6" si="2">E4+2</f>
+        <f t="shared" ref="E5:E6" si="3">E4+2</f>
         <v>5</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>336</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>87</v>
+        <v>328</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>328</v>
       </c>
       <c r="I5" s="98" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
       <c r="J5" s="98" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="K5" s="102"/>
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="16"/>
-      <c r="O5" s="35" t="s">
-        <v>339</v>
-      </c>
-      <c r="P5" s="5" t="s">
-        <v>340</v>
-      </c>
+      <c r="O5" s="35"/>
+      <c r="P5" s="5"/>
       <c r="Q5" s="5"/>
       <c r="R5" s="5"/>
       <c r="S5" s="16"/>
@@ -6721,10 +7539,10 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1">
       <c r="A6" s="75">
         <f>A5+14</f>
-        <v>46093</v>
+        <v>46457</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>190</v>
@@ -6738,31 +7556,27 @@
         <v>Thursday</v>
       </c>
       <c r="E6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>341</v>
+        <v>327</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>95</v>
+        <v>328</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>328</v>
       </c>
       <c r="I6" s="98" t="s">
-        <v>342</v>
+        <v>328</v>
       </c>
       <c r="J6" s="98" t="s">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="K6" s="102"/>
-      <c r="L6" s="24" t="s">
-        <v>344</v>
-      </c>
-      <c r="M6" s="24" t="s">
-        <v>345</v>
-      </c>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
       <c r="N6" s="16"/>
       <c r="O6" s="35"/>
       <c r="P6" s="5"/>
@@ -6776,47 +7590,44 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1">
       <c r="A7" s="75">
-        <f>A6+7</f>
-        <v>46100</v>
+        <f>A6+14</f>
+        <v>46471</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C7" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="D7" s="27" t="s">
-        <v>278</v>
+      <c r="C7" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v>Mar</v>
+      </c>
+      <c r="D7" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>Thursday</v>
       </c>
       <c r="E7">
-        <v>8</v>
+        <f>E6+2</f>
+        <v>9</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>346</v>
+        <v>327</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>101</v>
+        <v>328</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>328</v>
       </c>
       <c r="I7" s="98" t="s">
-        <v>347</v>
+        <v>328</v>
       </c>
       <c r="J7" s="98" t="s">
-        <v>348</v>
-      </c>
-      <c r="K7" s="102" t="s">
-        <v>349</v>
-      </c>
-      <c r="L7" s="24" t="s">
-        <v>350</v>
-      </c>
-      <c r="M7" s="24" t="s">
-        <v>351</v>
-      </c>
+        <v>328</v>
+      </c>
+      <c r="K7" s="102"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
       <c r="N7" s="16"/>
       <c r="O7" s="35"/>
       <c r="P7" s="5"/>
@@ -6830,49 +7641,45 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="17.25" customHeight="1">
       <c r="A8" s="75">
-        <f>A6+14</f>
-        <v>46107</v>
+        <f t="shared" ref="A8:A9" si="4">A7+14</f>
+        <v>46485</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C8" s="26" t="str">
-        <f t="shared" si="0"/>
-        <v>Mar</v>
+      <c r="C8" s="26" t="s">
+        <v>209</v>
       </c>
       <c r="D8" s="27" t="str">
         <f t="shared" si="1"/>
         <v>Thursday</v>
       </c>
       <c r="E8">
-        <f>E6+2</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>352</v>
+        <v>327</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>87</v>
+        <v>328</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>328</v>
       </c>
       <c r="I8" s="98" t="s">
-        <v>353</v>
+        <v>328</v>
       </c>
       <c r="J8" s="98" t="s">
-        <v>354</v>
+        <v>328</v>
       </c>
       <c r="K8" s="102"/>
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
       <c r="N8" s="16"/>
       <c r="O8" s="35"/>
-      <c r="P8" s="5" t="s">
-        <v>355</v>
-      </c>
+      <c r="P8" s="5"/>
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
       <c r="S8" s="16"/>
@@ -6883,47 +7690,41 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="18" customHeight="1">
       <c r="A9" s="75">
-        <f>A8+7</f>
-        <v>46114</v>
+        <f t="shared" si="4"/>
+        <v>46499</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>190</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>209</v>
+        <v>329</v>
       </c>
       <c r="D9" s="27" t="s">
         <v>278</v>
       </c>
       <c r="E9">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>356</v>
+        <v>327</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>322</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>101</v>
+        <v>328</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>328</v>
       </c>
       <c r="I9" s="98" t="s">
-        <v>357</v>
+        <v>328</v>
       </c>
       <c r="J9" s="98" t="s">
-        <v>358</v>
-      </c>
-      <c r="K9" s="102" t="s">
-        <v>359</v>
-      </c>
-      <c r="L9" s="24" t="s">
-        <v>360</v>
-      </c>
-      <c r="M9" s="24" t="s">
-        <v>361</v>
-      </c>
+        <v>328</v>
+      </c>
+      <c r="K9" s="102"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
       <c r="N9" s="16"/>
       <c r="O9" s="35"/>
       <c r="P9" s="5"/>
@@ -6937,7 +7738,562 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15" customHeight="1">
+      <c r="A10" s="26"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="X10" s="20"/>
+      <c r="Y10" s="18"/>
+    </row>
+    <row r="11" spans="1:25" ht="14.25" customHeight="1">
+      <c r="A11" s="26"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+    </row>
+    <row r="12" spans="1:25" ht="16.5" customHeight="1">
+      <c r="A12" s="26"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+    </row>
+    <row r="13" spans="1:25" ht="18.75" customHeight="1">
+      <c r="A13" s="26"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+    </row>
+    <row r="14" spans="1:25" ht="18.75" customHeight="1"/>
+    <row r="15" spans="1:25" ht="20.25" customHeight="1">
+      <c r="A15" s="26"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="J15" s="129"/>
+      <c r="K15" s="172"/>
+      <c r="X15" s="20"/>
+      <c r="Y15" s="18"/>
+    </row>
+    <row r="16" spans="1:25" ht="12.75" customHeight="1">
+      <c r="A16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="I16" s="129"/>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="26"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="26"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+    </row>
+  </sheetData>
+  <protectedRanges>
+    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A15:E18" name="Range3_1"/>
+    <protectedRange sqref="X15:Y15" name="Range8_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A3:E13" name="Range3_1_2"/>
+    <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="A2:L2 N2:Y2" name="Range4_1_3"/>
+    <protectedRange algorithmName="SHA-512" hashValue="B/N8xqtMc7pXr3rfrr4k91A6IFAPX6lxEHUr9qsJ3yHA+MBnFuw+x27DjsTYKp86iL5C7QQh1TPFTQHueWpZbw==" saltValue="c0IR/echnZmip5yS1t29Rw==" spinCount="100000" sqref="T3:T9" name="Range6_1_2"/>
+    <protectedRange algorithmName="SHA-512" hashValue="BKDH3ki5lE3XQdc5qZnIH6o8wW8E0PkHgMZFCkv/XYDEa+b/qenui0oReDIqPDXHceUVJ+rEgU3I9CDBHraDYg==" saltValue="ruXqG4NOhhm7cSLor8wHfw==" spinCount="100000" sqref="O2:O9" name="Range7_1_2"/>
+    <protectedRange sqref="X10:Y10 F3:Y9" name="Range8_1_2"/>
+    <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="M2" name="Range4_1_1_2"/>
+  </protectedRanges>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F62D4156-0A06-4DBF-B1E7-3E12580121CB}">
+  <sheetPr>
+    <tabColor theme="0"/>
+  </sheetPr>
+  <dimension ref="A1:Y18"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" customWidth="1"/>
+    <col min="6" max="6" width="33.42578125" customWidth="1"/>
+    <col min="7" max="7" width="30.85546875" customWidth="1"/>
+    <col min="8" max="8" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.85546875" customWidth="1"/>
+    <col min="11" max="11" width="20.42578125" customWidth="1"/>
+    <col min="12" max="13" width="12.5703125" customWidth="1"/>
+    <col min="14" max="14" width="43.140625" customWidth="1"/>
+    <col min="15" max="15" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="36.5703125" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="39" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="P1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="30">
+      <c r="A2" s="64" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="76" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="63" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="78" t="s">
+        <v>137</v>
+      </c>
+      <c r="E2" s="64" t="s">
+        <v>189</v>
+      </c>
+      <c r="F2" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="141" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="142" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="143" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="140" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" s="144" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" s="66" t="s">
+        <v>14</v>
+      </c>
+      <c r="M2" s="66" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" s="67" t="s">
+        <v>16</v>
+      </c>
+      <c r="O2" s="68" t="s">
+        <v>17</v>
+      </c>
+      <c r="P2" s="66" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q2" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="R2" s="66" t="s">
+        <v>20</v>
+      </c>
+      <c r="S2" s="67" t="s">
+        <v>21</v>
+      </c>
+      <c r="T2" s="69" t="s">
+        <v>22</v>
+      </c>
+      <c r="U2" s="67" t="s">
+        <v>23</v>
+      </c>
+      <c r="V2" s="65" t="s">
+        <v>24</v>
+      </c>
+      <c r="W2" s="66" t="s">
+        <v>138</v>
+      </c>
+      <c r="X2" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y2" s="70" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" ht="15" customHeight="1">
+      <c r="A3" s="75">
+        <v>46051</v>
+      </c>
+      <c r="B3" s="77" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="29" t="str">
+        <f>TEXT(A3, "mmm")</f>
+        <v>Jan</v>
+      </c>
+      <c r="D3" s="55" t="str">
+        <f>TEXT(A3, "dddd")</f>
+        <v>Thursday</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>330</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>331</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="I3" s="98" t="s">
+        <v>332</v>
+      </c>
+      <c r="J3" s="98" t="s">
+        <v>333</v>
+      </c>
+      <c r="K3" s="73"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="35"/>
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="40"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="35"/>
+      <c r="U3" s="40"/>
+      <c r="V3" s="40"/>
+      <c r="W3" s="40"/>
+      <c r="X3" s="46"/>
+      <c r="Y3" s="44"/>
+    </row>
+    <row r="4" spans="1:25" ht="15.75" customHeight="1">
+      <c r="A4" s="75">
+        <f>A3+12</f>
+        <v>46063</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C4" s="26" t="str">
+        <f t="shared" ref="C4:C10" si="0">TEXT(A4, "mmm")</f>
+        <v>Feb</v>
+      </c>
+      <c r="D4" s="27" t="str">
+        <f t="shared" ref="D4:D10" si="1">TEXT(A4, "dddd")</f>
+        <v>Tuesday</v>
+      </c>
+      <c r="E4">
+        <f>E3+2</f>
+        <v>3</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="98" t="s">
+        <v>336</v>
+      </c>
+      <c r="J4" s="98" t="s">
+        <v>337</v>
+      </c>
+      <c r="K4" s="102"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="16"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="5"/>
+      <c r="W4" s="5"/>
+      <c r="X4" s="15"/>
+      <c r="Y4" s="13"/>
+    </row>
+    <row r="5" spans="1:25" ht="18.75" customHeight="1">
+      <c r="A5" s="75">
+        <f>A4+16</f>
+        <v>46079</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C5" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v>Feb</v>
+      </c>
+      <c r="D5" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>Thursday</v>
+      </c>
+      <c r="E5">
+        <f t="shared" ref="E5:E6" si="2">E4+2</f>
+        <v>5</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>338</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>339</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" s="98" t="s">
+        <v>340</v>
+      </c>
+      <c r="J5" s="98" t="s">
+        <v>341</v>
+      </c>
+      <c r="K5" s="102"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="35" t="s">
+        <v>342</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="5"/>
+      <c r="S5" s="16"/>
+      <c r="T5" s="35"/>
+      <c r="U5" s="5"/>
+      <c r="V5" s="5"/>
+      <c r="W5" s="5"/>
+      <c r="X5" s="15"/>
+      <c r="Y5" s="13"/>
+    </row>
+    <row r="6" spans="1:25" ht="15.75" customHeight="1">
+      <c r="A6" s="75">
+        <f>A5+14</f>
+        <v>46093</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C6" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v>Mar</v>
+      </c>
+      <c r="D6" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>Thursday</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>344</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="I6" s="98" t="s">
+        <v>345</v>
+      </c>
+      <c r="J6" s="98" t="s">
+        <v>346</v>
+      </c>
+      <c r="K6" s="102"/>
+      <c r="L6" s="24" t="s">
+        <v>347</v>
+      </c>
+      <c r="M6" s="24" t="s">
+        <v>348</v>
+      </c>
+      <c r="N6" s="16"/>
+      <c r="O6" s="35"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="16"/>
+      <c r="T6" s="35"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="5"/>
+      <c r="X6" s="15"/>
+      <c r="Y6" s="13"/>
+    </row>
+    <row r="7" spans="1:25" ht="15.75" customHeight="1">
+      <c r="A7" s="75">
+        <f>A6+7</f>
+        <v>46100</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="E7">
+        <v>8</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="I7" s="98" t="s">
+        <v>350</v>
+      </c>
+      <c r="J7" s="98" t="s">
+        <v>351</v>
+      </c>
+      <c r="K7" s="102" t="s">
+        <v>352</v>
+      </c>
+      <c r="L7" s="24" t="s">
+        <v>353</v>
+      </c>
+      <c r="M7" s="24" t="s">
+        <v>354</v>
+      </c>
+      <c r="N7" s="16"/>
+      <c r="O7" s="35"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="16"/>
+      <c r="T7" s="35"/>
+      <c r="U7" s="5"/>
+      <c r="V7" s="5"/>
+      <c r="W7" s="5"/>
+      <c r="X7" s="15"/>
+      <c r="Y7" s="13"/>
+    </row>
+    <row r="8" spans="1:25" ht="17.25" customHeight="1">
+      <c r="A8" s="75">
+        <f>A6+14</f>
+        <v>46107</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C8" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v>Mar</v>
+      </c>
+      <c r="D8" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>Thursday</v>
+      </c>
+      <c r="E8">
+        <f>E6+2</f>
+        <v>9</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>355</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I8" s="98" t="s">
+        <v>356</v>
+      </c>
+      <c r="J8" s="98" t="s">
+        <v>357</v>
+      </c>
+      <c r="K8" s="102"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="35"/>
+      <c r="P8" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="16"/>
+      <c r="T8" s="35"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="5"/>
+      <c r="W8" s="5"/>
+      <c r="X8" s="15"/>
+      <c r="Y8" s="13"/>
+    </row>
+    <row r="9" spans="1:25" ht="18" customHeight="1">
+      <c r="A9" s="75">
+        <f>A8+7</f>
+        <v>46114</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>209</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="E9">
+        <v>10</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>322</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="I9" s="98" t="s">
+        <v>360</v>
+      </c>
+      <c r="J9" s="98" t="s">
+        <v>361</v>
+      </c>
+      <c r="K9" s="102" t="s">
+        <v>362</v>
+      </c>
+      <c r="L9" s="24" t="s">
+        <v>363</v>
+      </c>
+      <c r="M9" s="24" t="s">
+        <v>364</v>
+      </c>
+      <c r="N9" s="16"/>
+      <c r="O9" s="35"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="16"/>
+      <c r="T9" s="35"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+      <c r="X9" s="15"/>
+      <c r="Y9" s="13"/>
+    </row>
+    <row r="10" spans="1:25" ht="15" customHeight="1">
       <c r="A10" s="75">
         <v>46120</v>
       </c>
@@ -6956,7 +8312,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>77</v>
@@ -6965,10 +8321,10 @@
         <v>87</v>
       </c>
       <c r="I10" s="98" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="J10" s="98" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K10" s="102"/>
       <c r="L10" s="5"/>
@@ -6986,12 +8342,12 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="14.25" customHeight="1">
       <c r="A11" s="75">
         <v>46121</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="C11" s="26" t="s">
         <v>209</v>
@@ -7003,7 +8359,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>195</v>
@@ -7012,17 +8368,17 @@
         <v>87</v>
       </c>
       <c r="I11" s="98" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="J11" s="98" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="K11" s="102" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="24" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="N11" s="16"/>
       <c r="O11" s="35"/>
@@ -7037,7 +8393,7 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1">
       <c r="A12" s="75">
         <v>46128</v>
       </c>
@@ -7056,7 +8412,7 @@
         <v>12</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>195</v>
@@ -7065,17 +8421,17 @@
         <v>78</v>
       </c>
       <c r="I12" s="98" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="J12" s="98" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="K12" s="102" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="L12" s="5"/>
       <c r="M12" s="24" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="N12" s="16"/>
       <c r="O12" s="35"/>
@@ -7090,7 +8446,7 @@
       <c r="X12" s="15"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="18.75" customHeight="1">
       <c r="A13" s="75">
         <v>46135</v>
       </c>
@@ -7107,7 +8463,7 @@
         <v>13</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>73</v>
@@ -7116,10 +8472,10 @@
         <v>95</v>
       </c>
       <c r="I13" s="98" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="J13" s="98" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="K13" s="102"/>
       <c r="L13" s="5"/>
@@ -7137,7 +8493,7 @@
       <c r="X13" s="15"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="18.75" customHeight="1">
       <c r="A14" s="75">
         <v>46142</v>
       </c>
@@ -7145,7 +8501,7 @@
         <v>259</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
       <c r="D14" s="27" t="s">
         <v>278</v>
@@ -7154,26 +8510,26 @@
         <v>14</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="J14" s="107" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="K14" s="102" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="L14" s="14"/>
       <c r="M14" s="102" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="N14" s="14"/>
       <c r="O14" s="35"/>
@@ -7188,7 +8544,7 @@
       <c r="X14" s="15"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25" ht="20.25" customHeight="1" thickBot="1">
       <c r="A15" s="26">
         <v>46155</v>
       </c>
@@ -7196,76 +8552,76 @@
         <v>190</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
       <c r="D15" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="E15">
         <v>16</v>
       </c>
       <c r="F15" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="G15" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="H15" t="s">
         <v>40</v>
       </c>
       <c r="I15" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="J15" s="129" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="K15" s="172" t="s">
-        <v>445</v>
+        <v>393</v>
       </c>
       <c r="M15" t="s">
-        <v>446</v>
+        <v>394</v>
       </c>
       <c r="X15" s="20"/>
       <c r="Y15" s="18"/>
     </row>
-    <row r="16" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="12.75" customHeight="1">
       <c r="A16" s="26">
         <v>46176</v>
       </c>
       <c r="B16" t="s">
-        <v>447</v>
+        <v>395</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="D16" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="E16">
         <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="G16" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="H16" t="s">
         <v>224</v>
       </c>
       <c r="I16" s="129" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="J16" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
@@ -7301,722 +8657,215 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A33E49C-EC2E-42B7-80E4-DD607C0B7A89}">
-  <dimension ref="A1:Y13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.5703125" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="6" max="6" width="33.42578125" customWidth="1"/>
-    <col min="7" max="7" width="30.85546875" customWidth="1"/>
-    <col min="8" max="8" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="31.85546875" customWidth="1"/>
-    <col min="11" max="11" width="20.42578125" customWidth="1"/>
-    <col min="12" max="13" width="12.5703125" customWidth="1"/>
-    <col min="14" max="14" width="43.140625" customWidth="1"/>
-    <col min="15" max="15" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="36.5703125" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="39" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="P1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="64" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="76" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="63" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="78" t="s">
-        <v>137</v>
-      </c>
-      <c r="E2" s="64" t="s">
-        <v>189</v>
-      </c>
-      <c r="F2" s="140" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="141" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" s="142" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" s="143" t="s">
-        <v>11</v>
-      </c>
-      <c r="J2" s="140" t="s">
-        <v>12</v>
-      </c>
-      <c r="K2" s="144" t="s">
-        <v>13</v>
-      </c>
-      <c r="L2" s="66" t="s">
-        <v>14</v>
-      </c>
-      <c r="M2" s="66" t="s">
-        <v>15</v>
-      </c>
-      <c r="N2" s="67" t="s">
-        <v>16</v>
-      </c>
-      <c r="O2" s="68" t="s">
-        <v>17</v>
-      </c>
-      <c r="P2" s="66" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q2" s="65" t="s">
-        <v>19</v>
-      </c>
-      <c r="R2" s="66" t="s">
-        <v>20</v>
-      </c>
-      <c r="S2" s="67" t="s">
-        <v>21</v>
-      </c>
-      <c r="T2" s="69" t="s">
-        <v>22</v>
-      </c>
-      <c r="U2" s="67" t="s">
-        <v>23</v>
-      </c>
-      <c r="V2" s="65" t="s">
-        <v>24</v>
-      </c>
-      <c r="W2" s="66" t="s">
-        <v>138</v>
-      </c>
-      <c r="X2" s="70" t="s">
-        <v>26</v>
-      </c>
-      <c r="Y2" s="70" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75">
-        <v>46275</v>
-      </c>
-      <c r="B3" s="77" t="s">
-        <v>190</v>
-      </c>
-      <c r="C3" s="29" t="str">
-        <f>TEXT(A3, "mmm")</f>
-        <v>Sep</v>
-      </c>
-      <c r="D3" s="55" t="str">
-        <f>TEXT(A3, "dddd")</f>
-        <v>Thursday</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>396</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="I3" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="J3" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="K3" s="73"/>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="38"/>
-      <c r="O3" s="35"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40"/>
-      <c r="S3" s="38"/>
-      <c r="T3" s="35"/>
-      <c r="U3" s="40"/>
-      <c r="V3" s="40"/>
-      <c r="W3" s="40"/>
-      <c r="X3" s="46"/>
-      <c r="Y3" s="44"/>
-    </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="75">
-        <f>A3+14</f>
-        <v>46289</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C4" s="26" t="str">
-        <f t="shared" ref="C4:C7" si="0">TEXT(A4, "mmm")</f>
-        <v>Sep</v>
-      </c>
-      <c r="D4" s="27" t="str">
-        <f t="shared" ref="D4:D8" si="1">TEXT(A4, "dddd")</f>
-        <v>Thursday</v>
-      </c>
-      <c r="E4">
-        <f>E3+2</f>
-        <v>3</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>396</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>395</v>
-      </c>
-      <c r="I4" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="J4" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="K4" s="102"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="16"/>
-      <c r="O4" s="35"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="16"/>
-      <c r="T4" s="35"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="15"/>
-      <c r="Y4" s="13"/>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A5" s="75">
-        <f t="shared" ref="A5" si="2">A4+14</f>
-        <v>46303</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C5" s="26" t="str">
-        <f t="shared" si="0"/>
-        <v>Oct</v>
-      </c>
-      <c r="D5" s="27" t="str">
-        <f t="shared" si="1"/>
-        <v>Thursday</v>
-      </c>
-      <c r="E5">
-        <f t="shared" ref="E5:E6" si="3">E4+2</f>
-        <v>5</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>396</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="I5" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="J5" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="K5" s="102"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="35" t="s">
-        <v>339</v>
-      </c>
-      <c r="P5" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="16"/>
-      <c r="T5" s="35"/>
-      <c r="U5" s="5"/>
-      <c r="V5" s="5"/>
-      <c r="W5" s="5"/>
-      <c r="X5" s="15"/>
-      <c r="Y5" s="13"/>
-    </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="75">
-        <f>A5+14</f>
-        <v>46317</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C6" s="26" t="str">
-        <f t="shared" si="0"/>
-        <v>Oct</v>
-      </c>
-      <c r="D6" s="27" t="str">
-        <f t="shared" si="1"/>
-        <v>Thursday</v>
-      </c>
-      <c r="E6">
-        <f t="shared" si="3"/>
-        <v>7</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>396</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="I6" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="J6" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="K6" s="102"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="16"/>
-      <c r="O6" s="35"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="16"/>
-      <c r="T6" s="35"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
-      <c r="X6" s="15"/>
-      <c r="Y6" s="13"/>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="75">
-        <f>A6+14</f>
-        <v>46331</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C7" s="26" t="str">
-        <f t="shared" si="0"/>
-        <v>Nov</v>
-      </c>
-      <c r="D7" s="27" t="str">
-        <f t="shared" si="1"/>
-        <v>Thursday</v>
-      </c>
-      <c r="E7">
-        <f>E6+2</f>
-        <v>9</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>396</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="I7" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="J7" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="K7" s="102"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="35"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5"/>
-      <c r="R7" s="5"/>
-      <c r="S7" s="16"/>
-      <c r="T7" s="35"/>
-      <c r="U7" s="5"/>
-      <c r="V7" s="5"/>
-      <c r="W7" s="5"/>
-      <c r="X7" s="15"/>
-      <c r="Y7" s="13"/>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="75">
-        <f>A7+14</f>
-        <v>46345</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C8" s="26" t="s">
-        <v>209</v>
-      </c>
-      <c r="D8" s="27" t="str">
-        <f t="shared" si="1"/>
-        <v>Thursday</v>
-      </c>
-      <c r="E8">
-        <v>11</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>396</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="I8" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="J8" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="K8" s="102"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="35"/>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="5"/>
-      <c r="R8" s="5"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="35"/>
-      <c r="U8" s="5"/>
-      <c r="V8" s="5"/>
-      <c r="W8" s="5"/>
-      <c r="X8" s="15"/>
-      <c r="Y8" s="13"/>
-    </row>
-    <row r="9" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="75">
-        <v>46121</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>378</v>
-      </c>
-      <c r="D9" s="27" t="s">
-        <v>278</v>
-      </c>
-      <c r="E9">
-        <v>13</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>396</v>
-      </c>
-      <c r="G9" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="I9" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="J9" s="98" t="s">
-        <v>395</v>
-      </c>
-      <c r="K9" s="102"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="35"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="5"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="16"/>
-      <c r="T9" s="35"/>
-      <c r="U9" s="5"/>
-      <c r="V9" s="5"/>
-      <c r="W9" s="5"/>
-      <c r="X9" s="15"/>
-      <c r="Y9" s="13"/>
-    </row>
-    <row r="10" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="X10" s="20"/>
-      <c r="Y10" s="18"/>
-    </row>
-    <row r="11" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="26"/>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="26"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13" s="26"/>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-    </row>
-  </sheetData>
-  <protectedRanges>
-    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A3:E13" name="Range3_1"/>
-    <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="A2:L2 N2:Y2" name="Range4_1"/>
-    <protectedRange algorithmName="SHA-512" hashValue="B/N8xqtMc7pXr3rfrr4k91A6IFAPX6lxEHUr9qsJ3yHA+MBnFuw+x27DjsTYKp86iL5C7QQh1TPFTQHueWpZbw==" saltValue="c0IR/echnZmip5yS1t29Rw==" spinCount="100000" sqref="T3:T9" name="Range6_1"/>
-    <protectedRange algorithmName="SHA-512" hashValue="BKDH3ki5lE3XQdc5qZnIH6o8wW8E0PkHgMZFCkv/XYDEa+b/qenui0oReDIqPDXHceUVJ+rEgU3I9CDBHraDYg==" saltValue="ruXqG4NOhhm7cSLor8wHfw==" spinCount="100000" sqref="O2:O9" name="Range7_1"/>
-    <protectedRange sqref="X10:Y10 F3:Y9" name="Range8_1"/>
-    <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="M2" name="Range4_1_1"/>
-  </protectedRanges>
-  <phoneticPr fontId="10" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AEC079F-155A-491D-9189-1418FC903287}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.28515625" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" s="55" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="B2" s="54" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" s="136" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="B3" s="137"/>
       <c r="C3" s="138" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B4" s="52"/>
       <c r="C4" s="50" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" s="52" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="B5" s="52"/>
       <c r="C5" s="50" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="52" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="B6" s="52" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C6" s="50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" s="52" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="B7" s="52" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="C7" s="50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" s="52" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="C8" s="50" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" s="52" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="B9" s="52"/>
       <c r="C9" s="50"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" s="52" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" s="52" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="B11" s="52" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" s="52" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="B12" s="52" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" s="52" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="B13" s="52" t="s">
+        <v>425</v>
+      </c>
+      <c r="C13" s="50" t="s">
         <v>421</v>
       </c>
-      <c r="C13" s="50" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" s="52" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" s="52" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" s="137" t="s">
         <v>321</v>
       </c>
       <c r="B16" s="137" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="C16" s="139" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" s="137" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B17" s="137" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="C17" s="139" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" s="52" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C18" s="50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" s="53" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="B19" s="53" t="s">
         <v>230</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="B20" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -8029,27 +8878,27 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD19DE5-C22F-4D41-B540-76D70438E18B}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="6" max="6" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1">
       <c r="A1" s="135" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="131" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="C1" s="130" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="169">
         <v>46051</v>
       </c>
@@ -8057,14 +8906,14 @@
         <v>1</v>
       </c>
       <c r="C2" s="170" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="F2" s="75"/>
       <c r="G2" s="77"/>
       <c r="H2" s="29"/>
       <c r="I2" s="55"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9">
       <c r="A3" s="171">
         <f>A2+7</f>
         <v>46058</v>
@@ -8074,14 +8923,14 @@
         <v>2</v>
       </c>
       <c r="C3" s="170" t="s">
-        <v>396</v>
+        <v>327</v>
       </c>
       <c r="F3" s="75"/>
       <c r="G3" s="2"/>
       <c r="H3" s="26"/>
       <c r="I3" s="27"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9">
       <c r="A4" s="171">
         <f t="shared" ref="A4:A12" si="0">A3+7</f>
         <v>46065</v>
@@ -8091,14 +8940,14 @@
         <v>3</v>
       </c>
       <c r="C4" s="170" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="F4" s="75"/>
       <c r="G4" s="2"/>
       <c r="H4" s="26"/>
       <c r="I4" s="27"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9">
       <c r="A5" s="171">
         <f t="shared" si="0"/>
         <v>46072</v>
@@ -8108,14 +8957,14 @@
         <v>4</v>
       </c>
       <c r="C5" s="170" t="s">
-        <v>396</v>
+        <v>327</v>
       </c>
       <c r="F5" s="75"/>
       <c r="G5" s="2"/>
       <c r="H5" s="26"/>
       <c r="I5" s="27"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9">
       <c r="A6" s="133">
         <f t="shared" si="0"/>
         <v>46079</v>
@@ -8125,14 +8974,14 @@
         <v>5</v>
       </c>
       <c r="C6" s="134" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="F6" s="75"/>
       <c r="G6" s="2"/>
       <c r="H6" s="26"/>
       <c r="I6" s="27"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="A7" s="133">
         <f t="shared" si="0"/>
         <v>46086</v>
@@ -8142,14 +8991,14 @@
         <v>6</v>
       </c>
       <c r="C7" s="134" t="s">
-        <v>396</v>
+        <v>327</v>
       </c>
       <c r="F7" s="75"/>
       <c r="G7" s="2"/>
       <c r="H7" s="26"/>
       <c r="I7" s="27"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9">
       <c r="A8" s="133">
         <f t="shared" si="0"/>
         <v>46093</v>
@@ -8159,14 +9008,14 @@
         <v>7</v>
       </c>
       <c r="C8" s="134" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="F8" s="75"/>
       <c r="G8" s="2"/>
       <c r="H8" s="26"/>
       <c r="I8" s="27"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9">
       <c r="A9" s="133">
         <f t="shared" si="0"/>
         <v>46100</v>
@@ -8176,14 +9025,14 @@
         <v>8</v>
       </c>
       <c r="C9" s="134" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="F9" s="75"/>
       <c r="G9" s="2"/>
       <c r="H9" s="26"/>
       <c r="I9" s="27"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9">
       <c r="A10" s="133">
         <f t="shared" si="0"/>
         <v>46107</v>
@@ -8193,14 +9042,14 @@
         <v>9</v>
       </c>
       <c r="C10" s="134" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="F10" s="75"/>
       <c r="G10" s="2"/>
       <c r="H10" s="26"/>
       <c r="I10" s="27"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9">
       <c r="A11" s="133">
         <f t="shared" si="0"/>
         <v>46114</v>
@@ -8210,10 +9059,10 @@
         <v>10</v>
       </c>
       <c r="C11" s="134" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" s="133">
         <f t="shared" si="0"/>
         <v>46121</v>
@@ -8223,10 +9072,10 @@
         <v>11</v>
       </c>
       <c r="C12" s="134" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" s="133">
         <f t="shared" ref="A13:A14" si="3">A12+7</f>
         <v>46128</v>
@@ -8236,10 +9085,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="134" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14" s="133">
         <f t="shared" si="3"/>
         <v>46135</v>
@@ -8249,15 +9098,15 @@
         <v>13</v>
       </c>
       <c r="C14" s="134" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15" s="133"/>
       <c r="B15" s="134"/>
       <c r="C15" s="134"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9">
       <c r="G16" s="26"/>
     </row>
   </sheetData>
@@ -8279,319 +9128,4 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2BB5C5F-5790-4A91-A6E8-8841719DA1FC}">
-  <dimension ref="A2:I20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.7109375" customWidth="1"/>
-    <col min="7" max="7" width="38.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.42578125" customWidth="1"/>
-    <col min="9" max="9" width="64.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:9" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="91" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="79" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="80" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="80" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="80" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="80" t="s">
-        <v>137</v>
-      </c>
-      <c r="E5" s="80" t="s">
-        <v>189</v>
-      </c>
-      <c r="F5" s="80" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" s="80" t="s">
-        <v>9</v>
-      </c>
-      <c r="H5" s="82" t="s">
-        <v>440</v>
-      </c>
-      <c r="I5" s="81" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="92">
-        <v>45694</v>
-      </c>
-      <c r="B6" s="92" t="s">
-        <v>190</v>
-      </c>
-      <c r="C6" s="92" t="s">
-        <v>191</v>
-      </c>
-      <c r="D6" s="93" t="s">
-        <v>278</v>
-      </c>
-      <c r="E6" s="93">
-        <v>2</v>
-      </c>
-      <c r="F6" s="85" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="85" t="s">
-        <v>68</v>
-      </c>
-      <c r="H6" s="85"/>
-      <c r="I6" s="84" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="83">
-        <v>45708</v>
-      </c>
-      <c r="B7" s="83" t="s">
-        <v>190</v>
-      </c>
-      <c r="C7" s="83" t="s">
-        <v>191</v>
-      </c>
-      <c r="D7" s="94" t="s">
-        <v>278</v>
-      </c>
-      <c r="E7" s="94">
-        <v>4</v>
-      </c>
-      <c r="F7" s="87" t="s">
-        <v>194</v>
-      </c>
-      <c r="G7" s="87" t="s">
-        <v>195</v>
-      </c>
-      <c r="H7" s="87" t="s">
-        <v>78</v>
-      </c>
-      <c r="I7" s="86" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="83">
-        <v>45722</v>
-      </c>
-      <c r="B8" s="83" t="s">
-        <v>190</v>
-      </c>
-      <c r="C8" s="83" t="s">
-        <v>198</v>
-      </c>
-      <c r="D8" s="94" t="s">
-        <v>278</v>
-      </c>
-      <c r="E8" s="94">
-        <v>6</v>
-      </c>
-      <c r="F8" s="87" t="s">
-        <v>199</v>
-      </c>
-      <c r="G8" s="87" t="s">
-        <v>68</v>
-      </c>
-      <c r="H8" s="87" t="s">
-        <v>200</v>
-      </c>
-      <c r="I8" s="86"/>
-    </row>
-    <row r="9" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="83">
-        <v>45735</v>
-      </c>
-      <c r="B9" s="83" t="s">
-        <v>139</v>
-      </c>
-      <c r="C9" s="83" t="s">
-        <v>198</v>
-      </c>
-      <c r="D9" s="94" t="s">
-        <v>386</v>
-      </c>
-      <c r="E9" s="94">
-        <v>8</v>
-      </c>
-      <c r="F9" s="87" t="s">
-        <v>204</v>
-      </c>
-      <c r="G9" s="87" t="s">
-        <v>205</v>
-      </c>
-      <c r="H9" s="87" t="s">
-        <v>206</v>
-      </c>
-      <c r="I9" s="86" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="83">
-        <v>45744</v>
-      </c>
-      <c r="B10" s="83" t="s">
-        <v>190</v>
-      </c>
-      <c r="C10" s="83" t="s">
-        <v>198</v>
-      </c>
-      <c r="D10" s="94" t="s">
-        <v>214</v>
-      </c>
-      <c r="E10" s="94">
-        <v>9</v>
-      </c>
-      <c r="F10" s="87" t="s">
-        <v>222</v>
-      </c>
-      <c r="G10" s="87" t="s">
-        <v>223</v>
-      </c>
-      <c r="H10" s="87" t="s">
-        <v>224</v>
-      </c>
-      <c r="I10" s="86"/>
-    </row>
-    <row r="11" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A11" s="83">
-        <v>45750</v>
-      </c>
-      <c r="B11" s="83" t="s">
-        <v>190</v>
-      </c>
-      <c r="C11" s="83" t="s">
-        <v>209</v>
-      </c>
-      <c r="D11" s="94" t="s">
-        <v>278</v>
-      </c>
-      <c r="E11" s="94">
-        <v>10</v>
-      </c>
-      <c r="F11" s="87" t="s">
-        <v>441</v>
-      </c>
-      <c r="G11" s="87" t="s">
-        <v>68</v>
-      </c>
-      <c r="H11" s="87"/>
-      <c r="I11" s="86" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="83">
-        <v>45758</v>
-      </c>
-      <c r="B12" s="83" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="83" t="s">
-        <v>209</v>
-      </c>
-      <c r="D12" s="94" t="s">
-        <v>214</v>
-      </c>
-      <c r="E12" s="94">
-        <v>11</v>
-      </c>
-      <c r="F12" s="87" t="s">
-        <v>229</v>
-      </c>
-      <c r="G12" s="87" t="s">
-        <v>172</v>
-      </c>
-      <c r="H12" s="87" t="s">
-        <v>31</v>
-      </c>
-      <c r="I12" s="86" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A13" s="83">
-        <v>45764</v>
-      </c>
-      <c r="B13" s="83" t="s">
-        <v>190</v>
-      </c>
-      <c r="C13" s="83" t="s">
-        <v>209</v>
-      </c>
-      <c r="D13" s="94" t="s">
-        <v>278</v>
-      </c>
-      <c r="E13" s="94">
-        <v>12</v>
-      </c>
-      <c r="F13" s="87" t="s">
-        <v>442</v>
-      </c>
-      <c r="G13" s="87"/>
-      <c r="H13" s="87"/>
-      <c r="I13" s="86"/>
-    </row>
-    <row r="14" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A14" s="88">
-        <v>45771</v>
-      </c>
-      <c r="B14" s="88" t="s">
-        <v>190</v>
-      </c>
-      <c r="C14" s="88" t="s">
-        <v>209</v>
-      </c>
-      <c r="D14" s="95" t="s">
-        <v>278</v>
-      </c>
-      <c r="E14" s="95">
-        <v>13</v>
-      </c>
-      <c r="F14" s="90" t="s">
-        <v>443</v>
-      </c>
-      <c r="G14" s="90" t="s">
-        <v>77</v>
-      </c>
-      <c r="H14" s="90" t="s">
-        <v>124</v>
-      </c>
-      <c r="I14" s="89" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="20" spans="8:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="H20" s="79"/>
-    </row>
-  </sheetData>
-  <protectedRanges>
-    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A6:E13" name="Range3_1"/>
-    <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="A5:I5" name="Range4_1"/>
-    <protectedRange sqref="F6:I13" name="Range8_1"/>
-    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A14" name="Range3_3"/>
-  </protectedRanges>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
added title for MCS
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="558" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93651893-8D79-4E4A-BFD8-57E417923FD0}"/>
+  <xr:revisionPtr revIDLastSave="575" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDCAAB6C-A921-46CC-9709-3124C3A3A11C}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="21600" windowHeight="11175" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AY2023-2024 Sem 2" sheetId="3" state="hidden" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1136" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="473">
   <si>
     <t>Fill in as much of the green boxes as possible. Ideally, this would be before you have finished your visitors travel dates (just to avoid double booking).</t>
   </si>
@@ -1112,9 +1112,6 @@
     <t>David Osullivan</t>
   </si>
   <si>
-    <t xml:space="preserve"> Clustering smart meter electricity data in Ireland and the UK using functional data analysis</t>
-  </si>
-  <si>
     <t>https://www.linkedin.com/in/kate-finucane-997674151/</t>
   </si>
   <si>
@@ -1153,9 +1150,6 @@
     <t>https://scholar.google.com/citations?user=tXGb3D8AAAAJ&amp;hl=es</t>
   </si>
   <si>
-    <t>https://www.nature.com/articles/s42005-025-02406-5; https://arxiv.org/abs/2603.18801</t>
-  </si>
-  <si>
     <t>https://santiagolaot.github.io/ </t>
   </si>
   <si>
@@ -1517,6 +1511,30 @@
   </si>
   <si>
     <t>Leornard Henckel</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s42005-025-02406-5; https://journals.aps.org/prl/abstract/10.1103/56yd-sfks</t>
+  </si>
+  <si>
+    <t>Dec</t>
+  </si>
+  <si>
+    <t>Thomas Burnett</t>
+  </si>
+  <si>
+    <t>Eva Ryan</t>
+  </si>
+  <si>
+    <t>Making all pairwise comparisons in multi-arm clinical trials without control treatment</t>
+  </si>
+  <si>
+    <t>Clustering smart meter electricity data in Ireland and the UK using functional data analysis</t>
+  </si>
+  <si>
+    <t>Mathematical Modelling of Adsorption Columns State of the Art and Future Perspectives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column adsorption is an essential separation and purification process widely used in water treatment, greenhouse gas capture, air purification, and chromatography. While classical mathematical models for single-component systems under idealized conditions are well established, real-world applications present complex physical and chemical challenges that push standard models beyond their limitations. In this talk we provide a comprehensive overview of the current state of column adsorption modelling, focusing on recent theoretical advances that bridge the gap between simplified mathematical descriptions and realistic industrial environments. We will start from the general description for trace amounts, consisting of an advection-diffusion equation for mass transfer within the column and a kinetic equation for describing the adsorption mechanisms, and will discuss how this formulation is tweaked in different situations, such as the presence of large amounts of contaminant, consideration of multiple contaminant species to be removed simultaneously, increase of the size of the adsorbing particles, etc. </t>
   </si>
 </sst>
 </file>
@@ -1526,7 +1544,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2385,9 +2403,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2425,7 +2443,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2531,7 +2549,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2673,7 +2691,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2682,7 +2700,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7958562-D4BB-4776-9668-682A6F2E2AD0}">
   <dimension ref="A1:Y20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="11.140625" customWidth="1"/>
@@ -2707,7 +2725,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2718,7 +2736,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30">
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2795,7 +2813,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="13.5" customHeight="1">
+    <row r="3" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45317</v>
       </c>
@@ -2862,7 +2880,7 @@
       <c r="X3" s="13"/>
       <c r="Y3" s="13"/>
     </row>
-    <row r="4" spans="1:25" ht="13.5" customHeight="1">
+    <row r="4" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45323</v>
       </c>
@@ -2925,7 +2943,7 @@
       <c r="X4" s="13"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45324</v>
       </c>
@@ -2986,7 +3004,7 @@
       <c r="X5" s="13"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="12.75" customHeight="1">
+    <row r="6" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45331</v>
       </c>
@@ -3053,7 +3071,7 @@
       <c r="X6" s="13"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45338</v>
       </c>
@@ -3122,7 +3140,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1">
+    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45345</v>
       </c>
@@ -3189,7 +3207,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="16.5" customHeight="1">
+    <row r="9" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45359</v>
       </c>
@@ -3242,7 +3260,7 @@
       <c r="X9" s="13"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45366</v>
       </c>
@@ -3311,7 +3329,7 @@
       <c r="X10" s="13"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1">
+    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>45379</v>
       </c>
@@ -3372,7 +3390,7 @@
       <c r="X11" s="13"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="13.5" customHeight="1">
+    <row r="12" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>45386</v>
       </c>
@@ -3435,7 +3453,7 @@
       <c r="X12" s="13"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="16.5" customHeight="1">
+    <row r="13" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>45387</v>
       </c>
@@ -3504,7 +3522,7 @@
       <c r="X13" s="13"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>45394</v>
       </c>
@@ -3565,7 +3583,7 @@
       <c r="X14" s="13"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="17.25" customHeight="1">
+    <row r="15" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>45398</v>
       </c>
@@ -3634,7 +3652,7 @@
       <c r="X15" s="13"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>45401</v>
       </c>
@@ -3697,7 +3715,7 @@
       <c r="X16" s="18"/>
       <c r="Y16" s="18"/>
     </row>
-    <row r="17" spans="1:25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>45421</v>
       </c>
@@ -3768,7 +3786,7 @@
       <c r="X17" s="18"/>
       <c r="Y17" s="18"/>
     </row>
-    <row r="18" spans="1:25">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="26">
         <v>45474</v>
       </c>
@@ -3819,7 +3837,7 @@
       <c r="X18" s="18"/>
       <c r="Y18" s="18"/>
     </row>
-    <row r="19" spans="1:25" ht="17.25" customHeight="1" thickBot="1">
+    <row r="19" spans="1:25" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="26">
         <v>45505</v>
       </c>
@@ -3870,7 +3888,7 @@
       <c r="X19" s="18"/>
       <c r="Y19" s="18"/>
     </row>
-    <row r="20" spans="1:25">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="26"/>
       <c r="B20" s="26"/>
       <c r="C20" s="26"/>
@@ -3912,7 +3930,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2BB5C5F-5790-4A91-A6E8-8841719DA1FC}">
   <dimension ref="A2:I20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" customWidth="1"/>
     <col min="2" max="2" width="9.140625" customWidth="1"/>
@@ -3924,17 +3942,17 @@
     <col min="9" max="9" width="64.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" ht="23.25">
+    <row r="2" spans="1:9" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A2" s="91" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="18.75">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="79" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="37.5">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A5" s="80" t="s">
         <v>3</v>
       </c>
@@ -3957,13 +3975,13 @@
         <v>9</v>
       </c>
       <c r="H5" s="82" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="I5" s="81" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="18.75">
+    <row r="6" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="92">
         <v>45694</v>
       </c>
@@ -3990,7 +4008,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="18.75">
+    <row r="7" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="83">
         <v>45708</v>
       </c>
@@ -4019,7 +4037,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="18.75">
+    <row r="8" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="83">
         <v>45722</v>
       </c>
@@ -4046,7 +4064,7 @@
       </c>
       <c r="I8" s="86"/>
     </row>
-    <row r="9" spans="1:9" ht="18.75">
+    <row r="9" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="83">
         <v>45735</v>
       </c>
@@ -4057,7 +4075,7 @@
         <v>198</v>
       </c>
       <c r="D9" s="94" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="E9" s="94">
         <v>8</v>
@@ -4075,7 +4093,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="18.75">
+    <row r="10" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A10" s="83">
         <v>45744</v>
       </c>
@@ -4102,7 +4120,7 @@
       </c>
       <c r="I10" s="86"/>
     </row>
-    <row r="11" spans="1:9" ht="18.75">
+    <row r="11" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A11" s="83">
         <v>45750</v>
       </c>
@@ -4119,7 +4137,7 @@
         <v>10</v>
       </c>
       <c r="F11" s="87" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="G11" s="87" t="s">
         <v>68</v>
@@ -4129,7 +4147,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="18.75">
+    <row r="12" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="83">
         <v>45758</v>
       </c>
@@ -4158,7 +4176,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="18.75">
+    <row r="13" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="83">
         <v>45764</v>
       </c>
@@ -4175,13 +4193,13 @@
         <v>12</v>
       </c>
       <c r="F13" s="87" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="G13" s="87"/>
       <c r="H13" s="87"/>
       <c r="I13" s="86"/>
     </row>
-    <row r="14" spans="1:9" ht="18.75">
+    <row r="14" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="88">
         <v>45771</v>
       </c>
@@ -4198,7 +4216,7 @@
         <v>13</v>
       </c>
       <c r="F14" s="90" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="G14" s="90" t="s">
         <v>77</v>
@@ -4210,7 +4228,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="20" spans="8:8" ht="18.75">
+    <row r="20" spans="8:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="H20" s="79"/>
     </row>
   </sheetData>
@@ -4227,7 +4245,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y44"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="11.140625" customWidth="1"/>
@@ -4252,7 +4270,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4263,7 +4281,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30.75" thickBot="1">
+    <row r="2" spans="1:25" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="145" t="s">
         <v>3</v>
       </c>
@@ -4340,7 +4358,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45548</v>
       </c>
@@ -4405,7 +4423,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15" customHeight="1">
+    <row r="4" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45555</v>
       </c>
@@ -4454,7 +4472,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="15" customHeight="1">
+    <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45562</v>
       </c>
@@ -4503,7 +4521,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15" customHeight="1">
+    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45576</v>
       </c>
@@ -4552,7 +4570,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15" customHeight="1">
+    <row r="7" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45583</v>
       </c>
@@ -4601,7 +4619,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1">
+    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45596</v>
       </c>
@@ -4650,7 +4668,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15" customHeight="1">
+    <row r="9" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45604</v>
       </c>
@@ -4699,7 +4717,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1">
+    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45611</v>
       </c>
@@ -4748,7 +4766,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1">
+    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>45625</v>
       </c>
@@ -4797,7 +4815,7 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="15" customHeight="1" thickBot="1">
+    <row r="12" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>45632</v>
       </c>
@@ -4854,20 +4872,20 @@
       <c r="X12" s="20"/>
       <c r="Y12" s="18"/>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="26"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
       <c r="D13" s="26"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="26"/>
       <c r="B14" s="26"/>
       <c r="C14" s="26"/>
       <c r="D14" s="26"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -4879,59 +4897,59 @@
       <c r="I29" s="61"/>
       <c r="J29" s="61"/>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="60"/>
       <c r="B31" s="60"/>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="60"/>
       <c r="B32" s="60"/>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="60"/>
       <c r="B33" s="60"/>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="60"/>
       <c r="B34" s="60"/>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="60"/>
       <c r="B35" s="60"/>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="60"/>
       <c r="B36" s="60"/>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="60"/>
       <c r="B37" s="60"/>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="60"/>
       <c r="B38" s="60"/>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="60"/>
       <c r="B39" s="60"/>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="60"/>
       <c r="B40" s="60"/>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="60"/>
       <c r="B41" s="60"/>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="60"/>
       <c r="B42" s="60"/>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="60"/>
       <c r="B43" s="60"/>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="60"/>
       <c r="B44" s="60"/>
     </row>
@@ -4960,7 +4978,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12299A9A-6C0C-4F92-957E-FBFCB6211744}">
   <dimension ref="A1:Y45"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="5.85546875" bestFit="1" customWidth="1"/>
@@ -4988,7 +5006,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4999,7 +5017,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="27.75" customHeight="1" thickBot="1">
+    <row r="2" spans="1:25" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -5076,7 +5094,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45694</v>
       </c>
@@ -5128,7 +5146,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="14.25" customHeight="1">
+    <row r="4" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45708</v>
       </c>
@@ -5186,7 +5204,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="14.25" customHeight="1">
+    <row r="5" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45722</v>
       </c>
@@ -5242,7 +5260,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="16.5" customHeight="1">
+    <row r="6" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45735</v>
       </c>
@@ -5298,7 +5316,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="18" customHeight="1">
+    <row r="7" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45750</v>
       </c>
@@ -5352,7 +5370,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="16.5" customHeight="1">
+    <row r="8" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45751</v>
       </c>
@@ -5411,7 +5429,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45757</v>
       </c>
@@ -5473,7 +5491,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45758</v>
       </c>
@@ -5527,7 +5545,7 @@
       <c r="X10" s="20"/>
       <c r="Y10" s="18"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>45764</v>
       </c>
@@ -5587,7 +5605,7 @@
       <c r="X11" s="35"/>
       <c r="Y11" s="35"/>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>45771</v>
       </c>
@@ -5648,7 +5666,7 @@
       <c r="X12" s="35"/>
       <c r="Y12" s="35"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>45785</v>
       </c>
@@ -5701,7 +5719,7 @@
       <c r="X13" s="35"/>
       <c r="Y13" s="35"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>45799</v>
       </c>
@@ -5747,7 +5765,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>45805</v>
       </c>
@@ -5781,101 +5799,101 @@
         <v>250</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="75"/>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="26"/>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="26"/>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="26"/>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="75"/>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="26"/>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="75"/>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="26"/>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="26"/>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="26"/>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="26"/>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="26"/>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="26"/>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B31" s="60"/>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="60"/>
       <c r="B32" s="60"/>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="60"/>
       <c r="B33" s="60"/>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="60"/>
       <c r="B34" s="60"/>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="60"/>
       <c r="B35" s="60"/>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="60"/>
       <c r="B36" s="60"/>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="60"/>
       <c r="B37" s="60"/>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="60"/>
       <c r="B38" s="60"/>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="60"/>
       <c r="B39" s="60"/>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="60"/>
       <c r="B40" s="60"/>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="60"/>
       <c r="B41" s="60"/>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="60"/>
       <c r="B42" s="60"/>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="60"/>
       <c r="B43" s="60"/>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="60"/>
       <c r="B44" s="60"/>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="60"/>
     </row>
   </sheetData>
@@ -5900,7 +5918,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{243C2AD8-98F5-4435-96A3-1C2CAB922825}">
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
@@ -5927,7 +5945,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5938,7 +5956,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30">
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="78" t="s">
         <v>3</v>
       </c>
@@ -6015,7 +6033,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" thickBot="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="159">
         <v>45911</v>
       </c>
@@ -6078,7 +6096,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15" customHeight="1">
+    <row r="4" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="160">
         <v>45917</v>
       </c>
@@ -6147,7 +6165,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="15" customHeight="1">
+    <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="160">
         <v>45926</v>
       </c>
@@ -6205,7 +6223,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15" customHeight="1">
+    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="160">
         <v>45939</v>
       </c>
@@ -6269,7 +6287,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15" customHeight="1">
+    <row r="7" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="160">
         <v>45946</v>
       </c>
@@ -6326,7 +6344,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1">
+    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="160">
         <v>45953</v>
       </c>
@@ -6384,7 +6402,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15" customHeight="1">
+    <row r="9" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="160">
         <v>45967</v>
       </c>
@@ -6446,7 +6464,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1">
+    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="160">
         <v>45974</v>
       </c>
@@ -6509,7 +6527,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1">
+    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="160">
         <v>45980</v>
       </c>
@@ -6560,7 +6578,7 @@
       <c r="X11" s="35"/>
       <c r="Y11" s="35"/>
     </row>
-    <row r="12" spans="1:25" ht="16.5" customHeight="1">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="160">
         <f>A10+7</f>
         <v>45981</v>
@@ -6613,7 +6631,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="160">
         <v>45986</v>
       </c>
@@ -6649,7 +6667,7 @@
       <c r="M13" s="158"/>
       <c r="N13" s="158"/>
     </row>
-    <row r="14" spans="1:25" ht="15" customHeight="1">
+    <row r="14" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="160">
         <v>45988</v>
       </c>
@@ -6704,7 +6722,7 @@
       <c r="X14" s="15"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15" customHeight="1" thickBot="1">
+    <row r="15" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="161">
         <v>45995</v>
       </c>
@@ -6767,35 +6785,35 @@
       <c r="X15" s="15"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15" customHeight="1" thickBot="1">
+    <row r="16" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="26"/>
       <c r="B16" s="26"/>
       <c r="C16" s="26"/>
       <c r="X16" s="20"/>
       <c r="Y16" s="18"/>
     </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1">
+    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
     </row>
-    <row r="18" spans="1:3" ht="15" customHeight="1">
+    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
     </row>
-    <row r="19" spans="1:3" ht="15" customHeight="1">
+    <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="26"/>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
     </row>
-    <row r="20" spans="1:3" ht="15" customHeight="1"/>
-    <row r="21" spans="1:3" ht="15" customHeight="1"/>
-    <row r="22" spans="1:3" ht="15" customHeight="1"/>
-    <row r="23" spans="1:3" ht="15" customHeight="1"/>
-    <row r="24" spans="1:3" ht="15" customHeight="1"/>
-    <row r="25" spans="1:3" ht="15" customHeight="1"/>
-    <row r="26" spans="1:3" ht="15" customHeight="1"/>
+    <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <protectedRanges>
     <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A3:E19" name="Range3_1"/>
@@ -6828,8 +6846,8 @@
   <sheetPr>
     <tabColor rgb="FF00B050"/>
   </sheetPr>
-  <dimension ref="A1:Y15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:Y16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -6856,7 +6874,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="15.75" thickBot="1">
+    <row r="1" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6867,7 +6885,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30.75" thickBot="1">
+    <row r="2" spans="1:25" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -6944,7 +6962,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="75">
         <v>46275</v>
       </c>
@@ -6993,7 +7011,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="75">
         <f>A3+14</f>
         <v>46289</v>
@@ -7002,11 +7020,11 @@
         <v>190</v>
       </c>
       <c r="C4" s="26" t="str">
-        <f t="shared" ref="C4:C11" si="0">TEXT(A4, "mmm")</f>
+        <f t="shared" ref="C4:C12" si="0">TEXT(A4, "mmm")</f>
         <v>Sept</v>
       </c>
       <c r="D4" s="27" t="str">
-        <f t="shared" ref="D4:D10" si="1">TEXT(A4, "dddd")</f>
+        <f t="shared" ref="D4:D11" si="1">TEXT(A4, "dddd")</f>
         <v>Thursday</v>
       </c>
       <c r="E4">
@@ -7044,7 +7062,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="75">
         <f>A4+14</f>
         <v>46303</v>
@@ -7068,10 +7086,10 @@
         <v>329</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>330</v>
+        <v>77</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>331</v>
+        <v>31</v>
       </c>
       <c r="I5" s="98" t="s">
         <v>328</v>
@@ -7095,7 +7113,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="16.5" customHeight="1">
+    <row r="6" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="75">
         <v>46310</v>
       </c>
@@ -7123,7 +7141,7 @@
         <v>333</v>
       </c>
       <c r="I6" s="98" t="s">
-        <v>334</v>
+        <v>470</v>
       </c>
       <c r="J6" s="98" t="s">
         <v>328</v>
@@ -7131,7 +7149,7 @@
       <c r="K6" s="102"/>
       <c r="L6" s="5"/>
       <c r="M6" s="24" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="N6" s="16"/>
       <c r="O6" s="35"/>
@@ -7146,7 +7164,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="75">
         <f>A5+14</f>
         <v>46317</v>
@@ -7197,7 +7215,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15.75" customHeight="1">
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="75">
         <f>A7+7</f>
         <v>46324</v>
@@ -7217,26 +7235,26 @@
         <v>8</v>
       </c>
       <c r="F8" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>336</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="H8" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="I8" s="98" t="s">
+        <v>471</v>
+      </c>
+      <c r="J8" s="98" t="s">
+        <v>472</v>
+      </c>
+      <c r="K8" s="102" t="s">
         <v>338</v>
-      </c>
-      <c r="I8" s="98" t="s">
-        <v>328</v>
-      </c>
-      <c r="J8" s="98" t="s">
-        <v>328</v>
-      </c>
-      <c r="K8" s="102" t="s">
-        <v>339</v>
       </c>
       <c r="L8" s="5"/>
       <c r="M8" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="N8" s="16"/>
       <c r="O8" s="35"/>
@@ -7251,7 +7269,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="75">
         <f>A7+14</f>
         <v>46331</v>
@@ -7302,7 +7320,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="18.75" customHeight="1">
+    <row r="10" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="75">
         <f>A9+14</f>
         <v>46345</v>
@@ -7322,28 +7340,28 @@
         <v>11</v>
       </c>
       <c r="F10" s="16" t="s">
+        <v>340</v>
+      </c>
+      <c r="G10" s="14" t="s">
         <v>341</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>342</v>
       </c>
       <c r="H10" s="14" t="s">
         <v>333</v>
       </c>
       <c r="I10" s="98" t="s">
+        <v>342</v>
+      </c>
+      <c r="J10" s="98" t="s">
         <v>343</v>
       </c>
-      <c r="J10" s="98" t="s">
+      <c r="K10" s="102" t="s">
         <v>344</v>
       </c>
-      <c r="K10" s="102" t="s">
+      <c r="L10" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="M10" s="5" t="s">
         <v>345</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>347</v>
       </c>
       <c r="N10" s="16"/>
       <c r="O10" s="35"/>
@@ -7358,35 +7376,34 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="18.75" customHeight="1">
+    <row r="11" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="75">
-        <f>A10+14</f>
-        <v>46359</v>
+        <v>46357</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C11" s="26" t="str">
-        <f t="shared" si="0"/>
-        <v>Dec</v>
-      </c>
-      <c r="D11" s="27" t="s">
-        <v>278</v>
+      <c r="C11" s="26" t="s">
+        <v>466</v>
+      </c>
+      <c r="D11" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>Tuesday</v>
       </c>
       <c r="E11">
         <v>13</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>348</v>
+        <v>467</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>349</v>
+        <v>284</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>331</v>
+        <v>468</v>
       </c>
       <c r="I11" s="98" t="s">
-        <v>328</v>
+        <v>469</v>
       </c>
       <c r="J11" s="98" t="s">
         <v>328</v>
@@ -7407,35 +7424,84 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="15.75" thickBot="1">
-      <c r="A12" s="26"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="X12" s="20"/>
-      <c r="Y12" s="18"/>
-    </row>
-    <row r="13" spans="1:25" ht="12.75" customHeight="1">
+    <row r="12" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="75">
+        <f>A10+14</f>
+        <v>46359</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C12" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v>Dec</v>
+      </c>
+      <c r="D12" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="E12">
+        <v>13</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>346</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>347</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="I12" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="J12" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="K12" s="102"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="35"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="5"/>
+      <c r="S12" s="16"/>
+      <c r="T12" s="35"/>
+      <c r="U12" s="5"/>
+      <c r="V12" s="5"/>
+      <c r="W12" s="5"/>
+      <c r="X12" s="15"/>
+      <c r="Y12" s="13"/>
+    </row>
+    <row r="13" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="26"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
-    </row>
-    <row r="14" spans="1:25">
+      <c r="X13" s="20"/>
+      <c r="Y13" s="18"/>
+    </row>
+    <row r="14" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="26"/>
       <c r="B14" s="26"/>
       <c r="C14" s="26"/>
     </row>
-    <row r="15" spans="1:25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="26"/>
       <c r="B15" s="26"/>
       <c r="C15" s="26"/>
     </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A16" s="26"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+    </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A3:E15" name="Range3_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A3:E16" name="Range3_1"/>
     <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="A2:L2 N2:Y2" name="Range4_1"/>
-    <protectedRange algorithmName="SHA-512" hashValue="B/N8xqtMc7pXr3rfrr4k91A6IFAPX6lxEHUr9qsJ3yHA+MBnFuw+x27DjsTYKp86iL5C7QQh1TPFTQHueWpZbw==" saltValue="c0IR/echnZmip5yS1t29Rw==" spinCount="100000" sqref="T3:T11" name="Range6_1"/>
-    <protectedRange algorithmName="SHA-512" hashValue="BKDH3ki5lE3XQdc5qZnIH6o8wW8E0PkHgMZFCkv/XYDEa+b/qenui0oReDIqPDXHceUVJ+rEgU3I9CDBHraDYg==" saltValue="ruXqG4NOhhm7cSLor8wHfw==" spinCount="100000" sqref="O2:O11" name="Range7_1"/>
-    <protectedRange sqref="X12:Y12 F3:Y11" name="Range8_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="B/N8xqtMc7pXr3rfrr4k91A6IFAPX6lxEHUr9qsJ3yHA+MBnFuw+x27DjsTYKp86iL5C7QQh1TPFTQHueWpZbw==" saltValue="c0IR/echnZmip5yS1t29Rw==" spinCount="100000" sqref="T3:T12" name="Range6_1"/>
+    <protectedRange algorithmName="SHA-512" hashValue="BKDH3ki5lE3XQdc5qZnIH6o8wW8E0PkHgMZFCkv/XYDEa+b/qenui0oReDIqPDXHceUVJ+rEgU3I9CDBHraDYg==" saltValue="ruXqG4NOhhm7cSLor8wHfw==" spinCount="100000" sqref="O2:O12" name="Range7_1"/>
+    <protectedRange sqref="X13:Y13 F3:Y12" name="Range8_1"/>
     <protectedRange algorithmName="SHA-512" hashValue="JNB4nrqrfZD45ijUCOmyuk44ibTGOz2xPKKqUb8Fu6IzynfOW0Plt2J4MjvTXFpCm0cEkYqWWfoKwgUFnGztPw==" saltValue="gktf/myRKhBCN9s2pCislA==" spinCount="100000" sqref="M2" name="Range4_1_1"/>
   </protectedRanges>
   <phoneticPr fontId="10" type="noConversion"/>
@@ -7454,7 +7520,7 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:Y18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -7481,7 +7547,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7492,7 +7558,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30">
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -7569,7 +7635,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="75">
         <v>46415</v>
       </c>
@@ -7618,7 +7684,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="75">
         <f>A3+14</f>
         <v>46429</v>
@@ -7669,7 +7735,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="18.75" customHeight="1">
+    <row r="5" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="75">
         <f t="shared" ref="A5" si="2">A4+14</f>
         <v>46443</v>
@@ -7720,7 +7786,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="75">
         <f>A5+14</f>
         <v>46457</v>
@@ -7771,7 +7837,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="75">
         <f>A6+14</f>
         <v>46471</v>
@@ -7822,7 +7888,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="17.25" customHeight="1">
+    <row r="8" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="75">
         <f t="shared" ref="A8:A9" si="4">A7+14</f>
         <v>46485</v>
@@ -7871,7 +7937,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="18" customHeight="1">
+    <row r="9" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="75">
         <f t="shared" si="4"/>
         <v>46499</v>
@@ -7880,7 +7946,7 @@
         <v>190</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D9" s="27" t="s">
         <v>278</v>
@@ -7919,30 +7985,30 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1">
+    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26"/>
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
       <c r="X10" s="20"/>
       <c r="Y10" s="18"/>
     </row>
-    <row r="11" spans="1:25" ht="14.25" customHeight="1">
+    <row r="11" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="26"/>
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
     </row>
-    <row r="12" spans="1:25" ht="16.5" customHeight="1">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="26"/>
       <c r="B12" s="26"/>
       <c r="C12" s="26"/>
     </row>
-    <row r="13" spans="1:25" ht="18.75" customHeight="1">
+    <row r="13" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
     </row>
-    <row r="14" spans="1:25" ht="18.75" customHeight="1"/>
-    <row r="15" spans="1:25" ht="20.25" customHeight="1">
+    <row r="14" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:25" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26"/>
       <c r="B15" s="26"/>
       <c r="C15" s="26"/>
@@ -7951,17 +8017,17 @@
       <c r="X15" s="20"/>
       <c r="Y15" s="18"/>
     </row>
-    <row r="16" spans="1:25" ht="12.75" customHeight="1">
+    <row r="16" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="26"/>
       <c r="C16" s="26"/>
       <c r="I16" s="129"/>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
@@ -7985,7 +8051,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F62D4156-0A06-4DBF-B1E7-3E12580121CB}">
   <dimension ref="A1:Y18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -8012,7 +8078,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8023,7 +8089,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30">
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -8100,7 +8166,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="75">
         <v>46051</v>
       </c>
@@ -8119,19 +8185,19 @@
         <v>1</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>200</v>
       </c>
       <c r="I3" s="98" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="J3" s="98" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="K3" s="73"/>
       <c r="L3" s="40"/>
@@ -8149,13 +8215,13 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="75">
         <f>A3+12</f>
         <v>46063</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C4" s="26" t="str">
         <f t="shared" ref="C4:C10" si="0">TEXT(A4, "mmm")</f>
@@ -8170,7 +8236,7 @@
         <v>3</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="G4" s="16" t="s">
         <v>269</v>
@@ -8179,10 +8245,10 @@
         <v>87</v>
       </c>
       <c r="I4" s="98" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="J4" s="98" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="K4" s="102"/>
       <c r="L4" s="5"/>
@@ -8200,7 +8266,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="18.75" customHeight="1">
+    <row r="5" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="75">
         <f>A4+16</f>
         <v>46079</v>
@@ -8221,29 +8287,29 @@
         <v>5</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>87</v>
       </c>
       <c r="I5" s="98" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="J5" s="98" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="K5" s="102"/>
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="16"/>
       <c r="O5" s="35" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="Q5" s="5"/>
       <c r="R5" s="5"/>
@@ -8255,7 +8321,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="75">
         <f>A5+14</f>
         <v>46093</v>
@@ -8276,7 +8342,7 @@
         <v>7</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>152</v>
@@ -8285,17 +8351,17 @@
         <v>95</v>
       </c>
       <c r="I6" s="98" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="J6" s="98" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="K6" s="102"/>
       <c r="L6" s="24" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="M6" s="24" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="N6" s="16"/>
       <c r="O6" s="35"/>
@@ -8310,7 +8376,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="75">
         <f>A6+7</f>
         <v>46100</v>
@@ -8328,7 +8394,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="G7" s="14" t="s">
         <v>77</v>
@@ -8337,19 +8403,19 @@
         <v>101</v>
       </c>
       <c r="I7" s="98" t="s">
+        <v>369</v>
+      </c>
+      <c r="J7" s="98" t="s">
+        <v>370</v>
+      </c>
+      <c r="K7" s="102" t="s">
         <v>371</v>
       </c>
-      <c r="J7" s="98" t="s">
+      <c r="L7" s="24" t="s">
         <v>372</v>
       </c>
-      <c r="K7" s="102" t="s">
+      <c r="M7" s="24" t="s">
         <v>373</v>
-      </c>
-      <c r="L7" s="24" t="s">
-        <v>374</v>
-      </c>
-      <c r="M7" s="24" t="s">
-        <v>375</v>
       </c>
       <c r="N7" s="16"/>
       <c r="O7" s="35"/>
@@ -8364,7 +8430,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="17.25" customHeight="1">
+    <row r="8" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="75">
         <f>A6+14</f>
         <v>46107</v>
@@ -8385,7 +8451,7 @@
         <v>9</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="G8" s="14" t="s">
         <v>52</v>
@@ -8394,10 +8460,10 @@
         <v>87</v>
       </c>
       <c r="I8" s="98" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="J8" s="98" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="K8" s="102"/>
       <c r="L8" s="5"/>
@@ -8405,7 +8471,7 @@
       <c r="N8" s="16"/>
       <c r="O8" s="35"/>
       <c r="P8" s="5" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
@@ -8417,7 +8483,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="18" customHeight="1">
+    <row r="9" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="75">
         <f>A8+7</f>
         <v>46114</v>
@@ -8435,7 +8501,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>322</v>
@@ -8444,19 +8510,19 @@
         <v>101</v>
       </c>
       <c r="I9" s="98" t="s">
+        <v>379</v>
+      </c>
+      <c r="J9" s="98" t="s">
+        <v>380</v>
+      </c>
+      <c r="K9" s="102" t="s">
         <v>381</v>
       </c>
-      <c r="J9" s="98" t="s">
+      <c r="L9" s="24" t="s">
         <v>382</v>
       </c>
-      <c r="K9" s="102" t="s">
+      <c r="M9" s="24" t="s">
         <v>383</v>
-      </c>
-      <c r="L9" s="24" t="s">
-        <v>384</v>
-      </c>
-      <c r="M9" s="24" t="s">
-        <v>385</v>
       </c>
       <c r="N9" s="16"/>
       <c r="O9" s="35"/>
@@ -8471,7 +8537,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1">
+    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="75">
         <v>46120</v>
       </c>
@@ -8490,7 +8556,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>77</v>
@@ -8499,10 +8565,10 @@
         <v>87</v>
       </c>
       <c r="I10" s="98" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="J10" s="98" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K10" s="102"/>
       <c r="L10" s="5"/>
@@ -8520,12 +8586,12 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="14.25" customHeight="1">
+    <row r="11" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="75">
         <v>46121</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C11" s="26" t="s">
         <v>209</v>
@@ -8537,7 +8603,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>195</v>
@@ -8546,17 +8612,17 @@
         <v>87</v>
       </c>
       <c r="I11" s="98" t="s">
+        <v>388</v>
+      </c>
+      <c r="J11" s="98" t="s">
+        <v>389</v>
+      </c>
+      <c r="K11" s="102" t="s">
         <v>390</v>
-      </c>
-      <c r="J11" s="98" t="s">
-        <v>391</v>
-      </c>
-      <c r="K11" s="102" t="s">
-        <v>392</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="24" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="N11" s="16"/>
       <c r="O11" s="35"/>
@@ -8571,7 +8637,7 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="16.5" customHeight="1">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="75">
         <v>46128</v>
       </c>
@@ -8590,7 +8656,7 @@
         <v>12</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>195</v>
@@ -8599,17 +8665,17 @@
         <v>78</v>
       </c>
       <c r="I12" s="98" t="s">
+        <v>393</v>
+      </c>
+      <c r="J12" s="98" t="s">
+        <v>394</v>
+      </c>
+      <c r="K12" s="102" t="s">
         <v>395</v>
-      </c>
-      <c r="J12" s="98" t="s">
-        <v>396</v>
-      </c>
-      <c r="K12" s="102" t="s">
-        <v>397</v>
       </c>
       <c r="L12" s="5"/>
       <c r="M12" s="24" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="N12" s="16"/>
       <c r="O12" s="35"/>
@@ -8624,7 +8690,7 @@
       <c r="X12" s="15"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="18.75" customHeight="1">
+    <row r="13" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="75">
         <v>46135</v>
       </c>
@@ -8641,7 +8707,7 @@
         <v>13</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>73</v>
@@ -8650,10 +8716,10 @@
         <v>95</v>
       </c>
       <c r="I13" s="98" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="J13" s="98" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="K13" s="102"/>
       <c r="L13" s="5"/>
@@ -8671,7 +8737,7 @@
       <c r="X13" s="15"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="18.75" customHeight="1">
+    <row r="14" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="75">
         <v>46142</v>
       </c>
@@ -8679,7 +8745,7 @@
         <v>259</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D14" s="27" t="s">
         <v>278</v>
@@ -8688,26 +8754,26 @@
         <v>14</v>
       </c>
       <c r="F14" s="14" t="s">
+        <v>400</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="H14" s="14" t="s">
         <v>402</v>
       </c>
-      <c r="G14" s="14" t="s">
+      <c r="I14" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="J14" s="107" t="s">
         <v>404</v>
       </c>
-      <c r="I14" s="14" t="s">
+      <c r="K14" s="102" t="s">
         <v>405</v>
-      </c>
-      <c r="J14" s="107" t="s">
-        <v>406</v>
-      </c>
-      <c r="K14" s="102" t="s">
-        <v>407</v>
       </c>
       <c r="L14" s="14"/>
       <c r="M14" s="102" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="N14" s="14"/>
       <c r="O14" s="35"/>
@@ -8722,7 +8788,7 @@
       <c r="X14" s="15"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="20.25" customHeight="1" thickBot="1">
+    <row r="15" spans="1:25" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26">
         <v>46155</v>
       </c>
@@ -8730,76 +8796,76 @@
         <v>190</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D15" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="E15">
         <v>16</v>
       </c>
       <c r="F15" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="G15" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="H15" t="s">
         <v>40</v>
       </c>
       <c r="I15" t="s">
+        <v>410</v>
+      </c>
+      <c r="J15" s="129" t="s">
+        <v>411</v>
+      </c>
+      <c r="K15" s="172" t="s">
         <v>412</v>
       </c>
-      <c r="J15" s="129" t="s">
+      <c r="M15" t="s">
         <v>413</v>
-      </c>
-      <c r="K15" s="172" t="s">
-        <v>414</v>
-      </c>
-      <c r="M15" t="s">
-        <v>415</v>
       </c>
       <c r="X15" s="20"/>
       <c r="Y15" s="18"/>
     </row>
-    <row r="16" spans="1:25" ht="12.75" customHeight="1">
+    <row r="16" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="26">
         <v>46176</v>
       </c>
       <c r="B16" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D16" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="E16">
         <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="G16" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="H16" t="s">
         <v>224</v>
       </c>
       <c r="I16" s="129" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="J16" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
@@ -8838,212 +8904,212 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AEC079F-155A-491D-9189-1418FC903287}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.28515625" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="55" t="s">
+        <v>421</v>
+      </c>
+      <c r="B2" s="54" t="s">
         <v>422</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="55" t="s">
+      <c r="C2" s="54" t="s">
         <v>423</v>
       </c>
-      <c r="B2" s="54" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="136" t="s">
         <v>424</v>
-      </c>
-      <c r="C2" s="54" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="136" t="s">
-        <v>426</v>
       </c>
       <c r="B3" s="137"/>
       <c r="C3" s="138" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B4" s="52"/>
       <c r="C4" s="50" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="52" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B5" s="52"/>
       <c r="C5" s="50" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="52" t="s">
+        <v>428</v>
+      </c>
+      <c r="B6" s="52" t="s">
         <v>429</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="52" t="s">
-        <v>430</v>
-      </c>
-      <c r="B6" s="52" t="s">
-        <v>431</v>
       </c>
       <c r="C6" s="50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="52" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B7" s="52" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C7" s="50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="52" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C8" s="50" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B9" s="52"/>
       <c r="C9" s="50"/>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="52" t="s">
+        <v>435</v>
+      </c>
+      <c r="B10" s="52" t="s">
+        <v>436</v>
+      </c>
+      <c r="C10" s="50" t="s">
         <v>437</v>
       </c>
-      <c r="B10" s="52" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="52" t="s">
         <v>438</v>
       </c>
-      <c r="C10" s="50" t="s">
+      <c r="B11" s="52" t="s">
         <v>439</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="52" t="s">
-        <v>440</v>
-      </c>
-      <c r="B11" s="52" t="s">
-        <v>441</v>
       </c>
       <c r="C11" s="50" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="52" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B12" s="52" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="C12" s="50" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="52" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B13" s="52" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C13" s="50" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="52" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="C14" s="50" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="52" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C15" s="50" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="137" t="s">
         <v>321</v>
       </c>
       <c r="B16" s="137" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C16" s="139" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="137" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B17" s="137" t="s">
         <v>330</v>
       </c>
       <c r="C17" s="139" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="52" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C18" s="50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="53" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="B19" s="53" t="s">
         <v>230</v>
       </c>
       <c r="C19" s="51" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>453</v>
+      </c>
+      <c r="B20" t="s">
         <v>454</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
-        <v>455</v>
-      </c>
-      <c r="B20" t="s">
-        <v>456</v>
       </c>
     </row>
   </sheetData>
@@ -9059,24 +9125,24 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD19DE5-C22F-4D41-B540-76D70438E18B}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="6" max="6" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="135" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="131" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C1" s="130" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="169">
         <v>46051</v>
       </c>
@@ -9084,14 +9150,14 @@
         <v>1</v>
       </c>
       <c r="C2" s="170" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="F2" s="75"/>
       <c r="G2" s="77"/>
       <c r="H2" s="29"/>
       <c r="I2" s="55"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="171">
         <f>A2+7</f>
         <v>46058</v>
@@ -9108,7 +9174,7 @@
       <c r="H3" s="26"/>
       <c r="I3" s="27"/>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="171">
         <f t="shared" ref="A4:A12" si="0">A3+7</f>
         <v>46065</v>
@@ -9118,14 +9184,14 @@
         <v>3</v>
       </c>
       <c r="C4" s="170" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="F4" s="75"/>
       <c r="G4" s="2"/>
       <c r="H4" s="26"/>
       <c r="I4" s="27"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="171">
         <f t="shared" si="0"/>
         <v>46072</v>
@@ -9142,7 +9208,7 @@
       <c r="H5" s="26"/>
       <c r="I5" s="27"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="133">
         <f t="shared" si="0"/>
         <v>46079</v>
@@ -9152,14 +9218,14 @@
         <v>5</v>
       </c>
       <c r="C6" s="134" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="F6" s="75"/>
       <c r="G6" s="2"/>
       <c r="H6" s="26"/>
       <c r="I6" s="27"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="133">
         <f t="shared" si="0"/>
         <v>46086</v>
@@ -9176,7 +9242,7 @@
       <c r="H7" s="26"/>
       <c r="I7" s="27"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="133">
         <f t="shared" si="0"/>
         <v>46093</v>
@@ -9186,14 +9252,14 @@
         <v>7</v>
       </c>
       <c r="C8" s="134" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="F8" s="75"/>
       <c r="G8" s="2"/>
       <c r="H8" s="26"/>
       <c r="I8" s="27"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="133">
         <f t="shared" si="0"/>
         <v>46100</v>
@@ -9203,14 +9269,14 @@
         <v>8</v>
       </c>
       <c r="C9" s="134" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="F9" s="75"/>
       <c r="G9" s="2"/>
       <c r="H9" s="26"/>
       <c r="I9" s="27"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="133">
         <f t="shared" si="0"/>
         <v>46107</v>
@@ -9220,14 +9286,14 @@
         <v>9</v>
       </c>
       <c r="C10" s="134" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="F10" s="75"/>
       <c r="G10" s="2"/>
       <c r="H10" s="26"/>
       <c r="I10" s="27"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="133">
         <f t="shared" si="0"/>
         <v>46114</v>
@@ -9237,10 +9303,10 @@
         <v>10</v>
       </c>
       <c r="C11" s="134" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="133">
         <f t="shared" si="0"/>
         <v>46121</v>
@@ -9250,10 +9316,10 @@
         <v>11</v>
       </c>
       <c r="C12" s="134" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="133">
         <f t="shared" ref="A13:A14" si="3">A12+7</f>
         <v>46128</v>
@@ -9263,10 +9329,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="134" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="133">
         <f t="shared" si="3"/>
         <v>46135</v>
@@ -9276,15 +9342,15 @@
         <v>13</v>
       </c>
       <c r="C14" s="134" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="133"/>
       <c r="B15" s="134"/>
       <c r="C15" s="134"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="G16" s="26"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated with speakers abstract
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="575" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDCAAB6C-A921-46CC-9709-3124C3A3A11C}"/>
+  <xr:revisionPtr revIDLastSave="581" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6408A426-265A-4D5B-A9CB-7D7C421D3517}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AY2023-2024 Sem 2" sheetId="3" state="hidden" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="475">
   <si>
     <t>Fill in as much of the green boxes as possible. Ideally, this would be before you have finished your visitors travel dates (just to avoid double booking).</t>
   </si>
@@ -1535,6 +1535,12 @@
   </si>
   <si>
     <t xml:space="preserve">Column adsorption is an essential separation and purification process widely used in water treatment, greenhouse gas capture, air purification, and chromatography. While classical mathematical models for single-component systems under idealized conditions are well established, real-world applications present complex physical and chemical challenges that push standard models beyond their limitations. In this talk we provide a comprehensive overview of the current state of column adsorption modelling, focusing on recent theoretical advances that bridge the gap between simplified mathematical descriptions and realistic industrial environments. We will start from the general description for trace amounts, consisting of an advection-diffusion equation for mass transfer within the column and a kinetic equation for describing the adsorption mechanisms, and will discuss how this formulation is tweaked in different situations, such as the presence of large amounts of contaminant, consideration of multiple contaminant species to be removed simultaneously, increase of the size of the adsorbing particles, etc. </t>
+  </si>
+  <si>
+    <t>Generalised Linear Models Driven by Latent Processes: Asymptotic Theory and Applications</t>
+  </si>
+  <si>
+    <t>This paper introduces a class of generalised linear models (GLMs) driven by latent processes for modelling count, real-valued, binary, and positive continuous time series. Extending earlier latent-process regression frameworks based on Poisson or one-parameter exponential family assumptions, we allow the conditional distribution of the response to belong to a bi-parameter exponential family, with the latent process entering the conditional mean multiplicatively. This formulation substantially broadens the scope of latent-process GLMs, for instance, it naturally accommodates gamma responses for positive continuous data, enables estimation of an unknown dispersion parameter via the method of moments, and avoids restrictive conditions on link functions that arise under existing formulations. We establish the asymptotic normality of the GLM estimators obtained from the GLM likelihood that ignores the latent process, and we derive the correct information matrix for valid inference. In addition, we provide a principled approach to prediction and forecasting in GLMs driven by latent processes, a topic not previously addressed in the literature. We present two real data applications on measles infections in North Rhine-Westphalia (Germany) and paleoclimatic glacial varves, which highlight the practical advantages and enhanced flexibility of the proposed modelling framework.</t>
   </si>
 </sst>
 </file>
@@ -7062,7 +7068,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="75">
         <f>A4+14</f>
         <v>46303</v>
@@ -7092,10 +7098,10 @@
         <v>31</v>
       </c>
       <c r="I5" s="98" t="s">
-        <v>328</v>
+        <v>473</v>
       </c>
       <c r="J5" s="98" t="s">
-        <v>328</v>
+        <v>474</v>
       </c>
       <c r="K5" s="102"/>
       <c r="L5" s="5"/>

</xml_diff>